<commit_message>
chore: update selenium test report
</commit_message>
<xml_diff>
--- a/tests/reports/selenium-report.xlsx
+++ b/tests/reports/selenium-report.xlsx
@@ -40,7 +40,7 @@
     <t/>
   </si>
   <si>
-    <t>10/7/2026, 7:19:52 pm</t>
+    <t>11/7/2026, 10:07:22 pm</t>
   </si>
   <si>
     <t>TC002</t>
@@ -55,7 +55,7 @@
     <t>Login page shows ChemoSense branding</t>
   </si>
   <si>
-    <t>10/7/2026, 7:19:56 pm</t>
+    <t>11/7/2026, 10:07:26 pm</t>
   </si>
   <si>
     <t>TC004</t>
@@ -73,7 +73,7 @@
     <t>Invalid login shows error message</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:00 pm</t>
+    <t>11/7/2026, 10:07:29 pm</t>
   </si>
   <si>
     <t>TC006</t>
@@ -82,7 +82,7 @@
     <t>Demo login redirects to dashboard</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:10 pm</t>
+    <t>11/7/2026, 10:07:40 pm</t>
   </si>
   <si>
     <t>TC007</t>
@@ -118,7 +118,7 @@
     <t>Dashboard Total Scans card</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:14 pm</t>
+    <t>11/7/2026, 10:07:43 pm</t>
   </si>
   <si>
     <t>TC012</t>
@@ -163,6 +163,9 @@
     <t>Dashboard last cases shows real data</t>
   </si>
   <si>
+    <t>11/7/2026, 10:07:44 pm</t>
+  </si>
+  <si>
     <t>TC019</t>
   </si>
   <si>
@@ -181,7 +184,7 @@
     <t>Scan page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:17 pm</t>
+    <t>11/7/2026, 10:07:47 pm</t>
   </si>
   <si>
     <t>TC022</t>
@@ -208,16 +211,13 @@
     <t>Scan textarea accepts input</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:18 pm</t>
-  </si>
-  <si>
     <t>TC026</t>
   </si>
   <si>
     <t>Symptom scan returns AI results</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:31 pm</t>
+    <t>11/7/2026, 10:08:01 pm</t>
   </si>
   <si>
     <t>TC027</t>
@@ -256,7 +256,7 @@
     <t>Mode B biomarker mode works</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:36 pm</t>
+    <t>11/7/2026, 10:08:06 pm</t>
   </si>
   <si>
     <t>TC033</t>
@@ -265,7 +265,7 @@
     <t>Cases list page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:39 pm</t>
+    <t>11/7/2026, 10:08:09 pm</t>
   </si>
   <si>
     <t>TC034</t>
@@ -274,15 +274,15 @@
     <t>Cases shows total count</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:40 pm</t>
-  </si>
-  <si>
     <t>TC035</t>
   </si>
   <si>
     <t>Cases shows real database records</t>
   </si>
   <si>
+    <t>11/7/2026, 10:08:10 pm</t>
+  </si>
+  <si>
     <t>TC036</t>
   </si>
   <si>
@@ -307,7 +307,7 @@
     <t>Case detail page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:44 pm</t>
+    <t>11/7/2026, 10:08:13 pm</t>
   </si>
   <si>
     <t>TC040</t>
@@ -334,7 +334,7 @@
     <t>Patients page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:47 pm</t>
+    <t>11/7/2026, 10:08:17 pm</t>
   </si>
   <si>
     <t>TC044</t>
@@ -355,7 +355,7 @@
     <t>Patient selection shows timeline</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:50 pm</t>
+    <t>11/7/2026, 10:08:20 pm</t>
   </si>
   <si>
     <t>TC047</t>
@@ -376,7 +376,7 @@
     <t>Alerts page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:54 pm</t>
+    <t>11/7/2026, 10:08:23 pm</t>
   </si>
   <si>
     <t>TC050</t>
@@ -403,7 +403,7 @@
     <t>Bell icon links to alerts</t>
   </si>
   <si>
-    <t>10/7/2026, 7:20:57 pm</t>
+    <t>11/7/2026, 10:08:27 pm</t>
   </si>
   <si>
     <t>TC054</t>
@@ -412,7 +412,7 @@
     <t>Sensors page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:00 pm</t>
+    <t>11/7/2026, 10:08:30 pm</t>
   </si>
   <si>
     <t>TC055</t>
@@ -439,9 +439,6 @@
     <t>Sensor QS threshold visible</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:01 pm</t>
-  </si>
-  <si>
     <t>TC059</t>
   </si>
   <si>
@@ -472,7 +469,7 @@
     <t>Simulator page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:04 pm</t>
+    <t>11/7/2026, 10:08:34 pm</t>
   </si>
   <si>
     <t>TC064</t>
@@ -517,7 +514,7 @@
     <t>Simulator run scan generates live signal</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:14 pm</t>
+    <t>11/7/2026, 10:08:44 pm</t>
   </si>
   <si>
     <t>TC071</t>
@@ -526,7 +523,7 @@
     <t>Pathogen library loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:18 pm</t>
+    <t>11/7/2026, 10:08:47 pm</t>
   </si>
   <si>
     <t>TC072</t>
@@ -559,7 +556,7 @@
     <t>Pathogen detail page loads on click</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:20 pm</t>
+    <t>11/7/2026, 10:08:50 pm</t>
   </si>
   <si>
     <t>TC077</t>
@@ -568,7 +565,7 @@
     <t>Compare page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:24 pm</t>
+    <t>11/7/2026, 10:08:53 pm</t>
   </si>
   <si>
     <t>TC078</t>
@@ -583,6 +580,9 @@
     <t>Compare shows QS comparison</t>
   </si>
   <si>
+    <t>11/7/2026, 10:08:54 pm</t>
+  </si>
+  <si>
     <t>TC080</t>
   </si>
   <si>
@@ -595,7 +595,7 @@
     <t>Analytics page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:27 pm</t>
+    <t>11/7/2026, 10:08:57 pm</t>
   </si>
   <si>
     <t>TC082</t>
@@ -628,7 +628,7 @@
     <t>History page shows scan records</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:31 pm</t>
+    <t>11/7/2026, 10:09:00 pm</t>
   </si>
   <si>
     <t>TC087</t>
@@ -643,7 +643,7 @@
     <t>Outbreaks page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:34 pm</t>
+    <t>11/7/2026, 10:09:04 pm</t>
   </si>
   <si>
     <t>TC089</t>
@@ -658,7 +658,7 @@
     <t>Settings page loads</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:38 pm</t>
+    <t>11/7/2026, 10:09:07 pm</t>
   </si>
   <si>
     <t>TC091</t>
@@ -691,7 +691,7 @@
     <t>Backend health API healthy</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:40 pm</t>
+    <t>11/7/2026, 10:09:10 pm</t>
   </si>
   <si>
     <t>TC096</t>
@@ -700,7 +700,7 @@
     <t>Backend dashboard API returns stats</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:43 pm</t>
+    <t>11/7/2026, 10:09:13 pm</t>
   </si>
   <si>
     <t>TC097</t>
@@ -709,7 +709,7 @@
     <t>Backend scans API returns records</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:46 pm</t>
+    <t>11/7/2026, 10:09:17 pm</t>
   </si>
   <si>
     <t>TC098</t>
@@ -718,7 +718,7 @@
     <t>Backend patients API returns data</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:49 pm</t>
+    <t>11/7/2026, 10:09:20 pm</t>
   </si>
   <si>
     <t>TC099</t>
@@ -727,7 +727,7 @@
     <t>Backend outbreaks API returns data</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:51 pm</t>
+    <t>11/7/2026, 10:09:24 pm</t>
   </si>
   <si>
     <t>TC100</t>
@@ -736,7 +736,7 @@
     <t>Sign out redirects to login</t>
   </si>
   <si>
-    <t>10/7/2026, 7:21:58 pm</t>
+    <t>11/7/2026, 10:09:31 pm</t>
   </si>
   <si>
     <t>SUMMARY</t>
@@ -1484,32 +1484,32 @@
         <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>7</v>
@@ -1518,15 +1518,15 @@
         <v>8</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>7</v>
@@ -1535,32 +1535,32 @@
         <v>8</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>7</v>
@@ -1569,15 +1569,15 @@
         <v>8</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>7</v>
@@ -1586,15 +1586,15 @@
         <v>8</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>7</v>
@@ -1603,7 +1603,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1756,24 +1756,24 @@
         <v>8</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1790,7 +1790,7 @@
         <v>8</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1807,7 +1807,7 @@
         <v>8</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1824,7 +1824,7 @@
         <v>8</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2164,16 +2164,16 @@
         <v>8</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="C60" s="3" t="s">
         <v>7</v>
       </c>
@@ -2181,16 +2181,16 @@
         <v>8</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
     </row>
     <row r="61" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B61" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B61" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="C61" s="3" t="s">
         <v>7</v>
       </c>
@@ -2198,16 +2198,16 @@
         <v>8</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B62" s="2" t="s">
-        <v>148</v>
-      </c>
       <c r="C62" s="3" t="s">
         <v>7</v>
       </c>
@@ -2215,16 +2215,16 @@
         <v>8</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
     </row>
     <row r="63" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B63" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="C63" s="3" t="s">
         <v>7</v>
       </c>
@@ -2232,33 +2232,33 @@
         <v>8</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B64" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="C64" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="65" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B65" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B65" s="2" t="s">
-        <v>155</v>
-      </c>
       <c r="C65" s="3" t="s">
         <v>7</v>
       </c>
@@ -2266,16 +2266,16 @@
         <v>8</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B66" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="C66" s="3" t="s">
         <v>7</v>
       </c>
@@ -2283,16 +2283,16 @@
         <v>8</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B67" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B67" s="2" t="s">
-        <v>159</v>
-      </c>
       <c r="C67" s="3" t="s">
         <v>7</v>
       </c>
@@ -2300,16 +2300,16 @@
         <v>8</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B68" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B68" s="2" t="s">
-        <v>161</v>
-      </c>
       <c r="C68" s="3" t="s">
         <v>7</v>
       </c>
@@ -2317,16 +2317,16 @@
         <v>8</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B69" s="2" t="s">
-        <v>163</v>
-      </c>
       <c r="C69" s="3" t="s">
         <v>7</v>
       </c>
@@ -2334,16 +2334,16 @@
         <v>8</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B70" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B70" s="2" t="s">
-        <v>165</v>
-      </c>
       <c r="C70" s="3" t="s">
         <v>7</v>
       </c>
@@ -2351,50 +2351,50 @@
         <v>8</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B71" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="C71" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B72" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="C72" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E72" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B73" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B73" s="2" t="s">
-        <v>173</v>
-      </c>
       <c r="C73" s="3" t="s">
         <v>7</v>
       </c>
@@ -2402,16 +2402,16 @@
         <v>8</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B74" s="2" t="s">
-        <v>175</v>
-      </c>
       <c r="C74" s="3" t="s">
         <v>7</v>
       </c>
@@ -2419,16 +2419,16 @@
         <v>8</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B75" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="B75" s="2" t="s">
-        <v>177</v>
-      </c>
       <c r="C75" s="3" t="s">
         <v>7</v>
       </c>
@@ -2436,16 +2436,16 @@
         <v>8</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B76" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B76" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="C76" s="3" t="s">
         <v>7</v>
       </c>
@@ -2453,50 +2453,50 @@
         <v>8</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="C77" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E77" s="2" t="s">
         <v>181</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B78" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="C78" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E78" s="2" t="s">
         <v>184</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B79" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="B79" s="2" t="s">
-        <v>187</v>
-      </c>
       <c r="C79" s="3" t="s">
         <v>7</v>
       </c>
@@ -2504,24 +2504,24 @@
         <v>8</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="80" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="C80" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E80" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2538,7 +2538,7 @@
         <v>8</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
     <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: AI-powered pathogen comparison and Q&A
</commit_message>
<xml_diff>
--- a/tests/reports/selenium-report.xlsx
+++ b/tests/reports/selenium-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="246">
   <si>
     <t>Test ID</t>
   </si>
@@ -40,7 +40,7 @@
     <t/>
   </si>
   <si>
-    <t>11/7/2026, 10:07:22 pm</t>
+    <t>12/7/2026, 10:01:11 pm</t>
   </si>
   <si>
     <t>TC002</t>
@@ -55,7 +55,7 @@
     <t>Login page shows ChemoSense branding</t>
   </si>
   <si>
-    <t>11/7/2026, 10:07:26 pm</t>
+    <t>12/7/2026, 10:01:15 pm</t>
   </si>
   <si>
     <t>TC004</t>
@@ -73,7 +73,7 @@
     <t>Invalid login shows error message</t>
   </si>
   <si>
-    <t>11/7/2026, 10:07:29 pm</t>
+    <t>12/7/2026, 10:01:18 pm</t>
   </si>
   <si>
     <t>TC006</t>
@@ -82,7 +82,7 @@
     <t>Demo login redirects to dashboard</t>
   </si>
   <si>
-    <t>11/7/2026, 10:07:40 pm</t>
+    <t>12/7/2026, 10:01:28 pm</t>
   </si>
   <si>
     <t>TC007</t>
@@ -91,6 +91,9 @@
     <t>Dashboard visible after demo login</t>
   </si>
   <si>
+    <t>12/7/2026, 10:01:29 pm</t>
+  </si>
+  <si>
     <t>TC008</t>
   </si>
   <si>
@@ -118,7 +121,7 @@
     <t>Dashboard Total Scans card</t>
   </si>
   <si>
-    <t>11/7/2026, 10:07:43 pm</t>
+    <t>12/7/2026, 10:01:32 pm</t>
   </si>
   <si>
     <t>TC012</t>
@@ -163,9 +166,6 @@
     <t>Dashboard last cases shows real data</t>
   </si>
   <si>
-    <t>11/7/2026, 10:07:44 pm</t>
-  </si>
-  <si>
     <t>TC019</t>
   </si>
   <si>
@@ -184,7 +184,7 @@
     <t>Scan page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:07:47 pm</t>
+    <t>12/7/2026, 10:01:36 pm</t>
   </si>
   <si>
     <t>TC022</t>
@@ -217,7 +217,7 @@
     <t>Symptom scan returns AI results</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:01 pm</t>
+    <t>12/7/2026, 10:01:50 pm</t>
   </si>
   <si>
     <t>TC027</t>
@@ -256,7 +256,7 @@
     <t>Mode B biomarker mode works</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:06 pm</t>
+    <t>12/7/2026, 10:01:55 pm</t>
   </si>
   <si>
     <t>TC033</t>
@@ -265,7 +265,7 @@
     <t>Cases list page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:09 pm</t>
+    <t>12/7/2026, 10:01:58 pm</t>
   </si>
   <si>
     <t>TC034</t>
@@ -280,9 +280,6 @@
     <t>Cases shows real database records</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:10 pm</t>
-  </si>
-  <si>
     <t>TC036</t>
   </si>
   <si>
@@ -301,13 +298,16 @@
     <t>Cases shows risk level pills</t>
   </si>
   <si>
+    <t>12/7/2026, 10:01:59 pm</t>
+  </si>
+  <si>
     <t>TC039</t>
   </si>
   <si>
     <t>Case detail page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:13 pm</t>
+    <t>12/7/2026, 10:02:02 pm</t>
   </si>
   <si>
     <t>TC040</t>
@@ -334,7 +334,7 @@
     <t>Patients page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:17 pm</t>
+    <t>12/7/2026, 10:02:06 pm</t>
   </si>
   <si>
     <t>TC044</t>
@@ -355,7 +355,7 @@
     <t>Patient selection shows timeline</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:20 pm</t>
+    <t>12/7/2026, 10:02:09 pm</t>
   </si>
   <si>
     <t>TC047</t>
@@ -376,7 +376,7 @@
     <t>Alerts page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:23 pm</t>
+    <t>12/7/2026, 10:02:12 pm</t>
   </si>
   <si>
     <t>TC050</t>
@@ -403,7 +403,7 @@
     <t>Bell icon links to alerts</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:27 pm</t>
+    <t>12/7/2026, 10:02:16 pm</t>
   </si>
   <si>
     <t>TC054</t>
@@ -412,7 +412,7 @@
     <t>Sensors page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:30 pm</t>
+    <t>12/7/2026, 10:02:20 pm</t>
   </si>
   <si>
     <t>TC055</t>
@@ -469,7 +469,7 @@
     <t>Simulator page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:34 pm</t>
+    <t>12/7/2026, 10:02:23 pm</t>
   </si>
   <si>
     <t>TC064</t>
@@ -514,7 +514,7 @@
     <t>Simulator run scan generates live signal</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:44 pm</t>
+    <t>12/7/2026, 10:02:33 pm</t>
   </si>
   <si>
     <t>TC071</t>
@@ -523,7 +523,7 @@
     <t>Pathogen library loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:47 pm</t>
+    <t>12/7/2026, 10:02:37 pm</t>
   </si>
   <si>
     <t>TC072</t>
@@ -556,7 +556,7 @@
     <t>Pathogen detail page loads on click</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:50 pm</t>
+    <t>12/7/2026, 10:02:40 pm</t>
   </si>
   <si>
     <t>TC077</t>
@@ -565,7 +565,7 @@
     <t>Compare page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:53 pm</t>
+    <t>12/7/2026, 10:02:43 pm</t>
   </si>
   <si>
     <t>TC078</t>
@@ -580,9 +580,6 @@
     <t>Compare shows QS comparison</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:54 pm</t>
-  </si>
-  <si>
     <t>TC080</t>
   </si>
   <si>
@@ -595,7 +592,7 @@
     <t>Analytics page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:08:57 pm</t>
+    <t>12/7/2026, 10:02:47 pm</t>
   </si>
   <si>
     <t>TC082</t>
@@ -628,7 +625,7 @@
     <t>History page shows scan records</t>
   </si>
   <si>
-    <t>11/7/2026, 10:09:00 pm</t>
+    <t>12/7/2026, 10:02:50 pm</t>
   </si>
   <si>
     <t>TC087</t>
@@ -643,7 +640,7 @@
     <t>Outbreaks page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:09:04 pm</t>
+    <t>12/7/2026, 10:02:54 pm</t>
   </si>
   <si>
     <t>TC089</t>
@@ -658,7 +655,7 @@
     <t>Settings page loads</t>
   </si>
   <si>
-    <t>11/7/2026, 10:09:07 pm</t>
+    <t>12/7/2026, 10:02:57 pm</t>
   </si>
   <si>
     <t>TC091</t>
@@ -691,7 +688,7 @@
     <t>Backend health API healthy</t>
   </si>
   <si>
-    <t>11/7/2026, 10:09:10 pm</t>
+    <t>12/7/2026, 10:03:00 pm</t>
   </si>
   <si>
     <t>TC096</t>
@@ -700,7 +697,7 @@
     <t>Backend dashboard API returns stats</t>
   </si>
   <si>
-    <t>11/7/2026, 10:09:13 pm</t>
+    <t>12/7/2026, 10:03:04 pm</t>
   </si>
   <si>
     <t>TC097</t>
@@ -709,7 +706,7 @@
     <t>Backend scans API returns records</t>
   </si>
   <si>
-    <t>11/7/2026, 10:09:17 pm</t>
+    <t>12/7/2026, 10:03:08 pm</t>
   </si>
   <si>
     <t>TC098</t>
@@ -718,7 +715,7 @@
     <t>Backend patients API returns data</t>
   </si>
   <si>
-    <t>11/7/2026, 10:09:20 pm</t>
+    <t>12/7/2026, 10:03:12 pm</t>
   </si>
   <si>
     <t>TC099</t>
@@ -727,7 +724,7 @@
     <t>Backend outbreaks API returns data</t>
   </si>
   <si>
-    <t>11/7/2026, 10:09:24 pm</t>
+    <t>12/7/2026, 10:03:14 pm</t>
   </si>
   <si>
     <t>TC100</t>
@@ -736,7 +733,7 @@
     <t>Sign out redirects to login</t>
   </si>
   <si>
-    <t>11/7/2026, 10:09:31 pm</t>
+    <t>12/7/2026, 10:03:21 pm</t>
   </si>
   <si>
     <t>SUMMARY</t>
@@ -1297,49 +1294,49 @@
         <v>8</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>7</v>
@@ -1348,15 +1345,15 @@
         <v>8</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>7</v>
@@ -1365,32 +1362,32 @@
         <v>8</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>7</v>
@@ -1399,15 +1396,15 @@
         <v>8</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>7</v>
@@ -1416,15 +1413,15 @@
         <v>8</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>7</v>
@@ -1433,15 +1430,15 @@
         <v>8</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>7</v>
@@ -1450,15 +1447,15 @@
         <v>8</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>7</v>
@@ -1467,15 +1464,15 @@
         <v>8</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>7</v>
@@ -1484,7 +1481,7 @@
         <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1501,7 +1498,7 @@
         <v>8</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1518,7 +1515,7 @@
         <v>8</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1773,16 +1770,16 @@
         <v>8</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="C37" s="3" t="s">
         <v>7</v>
       </c>
@@ -1790,16 +1787,16 @@
         <v>8</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>93</v>
-      </c>
       <c r="C38" s="3" t="s">
         <v>7</v>
       </c>
@@ -1807,24 +1804,24 @@
         <v>8</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C39" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2521,16 +2518,16 @@
         <v>8</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="B81" s="2" t="s">
-        <v>191</v>
-      </c>
       <c r="C81" s="3" t="s">
         <v>7</v>
       </c>
@@ -2538,33 +2535,33 @@
         <v>8</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B82" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="C82" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E82" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="C82" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="83" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B83" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B83" s="2" t="s">
-        <v>196</v>
-      </c>
       <c r="C83" s="3" t="s">
         <v>7</v>
       </c>
@@ -2572,16 +2569,16 @@
         <v>8</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="84" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B84" s="2" t="s">
-        <v>198</v>
-      </c>
       <c r="C84" s="3" t="s">
         <v>7</v>
       </c>
@@ -2589,16 +2586,16 @@
         <v>8</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="85" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B85" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>200</v>
-      </c>
       <c r="C85" s="3" t="s">
         <v>7</v>
       </c>
@@ -2606,16 +2603,16 @@
         <v>8</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="86" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B86" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B86" s="2" t="s">
-        <v>202</v>
-      </c>
       <c r="C86" s="3" t="s">
         <v>7</v>
       </c>
@@ -2623,33 +2620,33 @@
         <v>8</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="87" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B87" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="C87" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E87" s="2" t="s">
         <v>204</v>
-      </c>
-      <c r="C87" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="88" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="B88" s="2" t="s">
-        <v>207</v>
-      </c>
       <c r="C88" s="3" t="s">
         <v>7</v>
       </c>
@@ -2657,33 +2654,33 @@
         <v>8</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="89" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B89" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="C89" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E89" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="90" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B90" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="B90" s="2" t="s">
-        <v>212</v>
-      </c>
       <c r="C90" s="3" t="s">
         <v>7</v>
       </c>
@@ -2691,33 +2688,33 @@
         <v>8</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="91" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B91" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B91" s="2" t="s">
+      <c r="C91" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E91" s="2" t="s">
         <v>214</v>
-      </c>
-      <c r="C91" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="92" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B92" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B92" s="2" t="s">
-        <v>217</v>
-      </c>
       <c r="C92" s="3" t="s">
         <v>7</v>
       </c>
@@ -2725,16 +2722,16 @@
         <v>8</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="93" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B93" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B93" s="2" t="s">
-        <v>219</v>
-      </c>
       <c r="C93" s="3" t="s">
         <v>7</v>
       </c>
@@ -2742,16 +2739,16 @@
         <v>8</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="94" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B94" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="B94" s="2" t="s">
-        <v>221</v>
-      </c>
       <c r="C94" s="3" t="s">
         <v>7</v>
       </c>
@@ -2759,16 +2756,16 @@
         <v>8</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="95" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B95" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B95" s="2" t="s">
-        <v>223</v>
-      </c>
       <c r="C95" s="3" t="s">
         <v>7</v>
       </c>
@@ -2776,126 +2773,126 @@
         <v>8</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="96" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B96" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="C96" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E96" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E96" s="2" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="97" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B97" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="C97" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E97" s="2" t="s">
         <v>228</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D97" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E97" s="2" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="98" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B98" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="C98" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E98" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="C98" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E98" s="2" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="99" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B99" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="C99" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E99" s="2" t="s">
         <v>234</v>
-      </c>
-      <c r="C99" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E99" s="2" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="100" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B100" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="B100" s="2" t="s">
+      <c r="C100" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E100" s="2" t="s">
         <v>237</v>
-      </c>
-      <c r="C100" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D100" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E100" s="2" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="101" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B101" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="C101" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E101" s="2" t="s">
         <v>240</v>
-      </c>
-      <c r="C101" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D101" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E101" s="2" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="103" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B103" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="B103" s="4" t="s">
+      <c r="C103" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="C103" s="4" t="s">
+      <c r="D103" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="D103" s="4" t="s">
+      <c r="E103" s="4" t="s">
         <v>245</v>
-      </c>
-      <c r="E103" s="4" t="s">
-        <v>246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: compare/pathogen-ask use full backend URL and unwrap Response
</commit_message>
<xml_diff>
--- a/tests/reports/selenium-report.xlsx
+++ b/tests/reports/selenium-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="434">
   <si>
     <t>Test ID</t>
   </si>
@@ -40,7 +40,7 @@
     <t/>
   </si>
   <si>
-    <t>12/7/2026, 10:01:11 pm</t>
+    <t>13/7/2026, 9:21:09 am</t>
   </si>
   <si>
     <t>TC002</t>
@@ -55,7 +55,7 @@
     <t>Login page shows ChemoSense branding</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:15 pm</t>
+    <t>13/7/2026, 9:21:13 am</t>
   </si>
   <si>
     <t>TC004</t>
@@ -73,7 +73,7 @@
     <t>Invalid login shows error message</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:18 pm</t>
+    <t>13/7/2026, 9:21:16 am</t>
   </si>
   <si>
     <t>TC006</t>
@@ -82,7 +82,7 @@
     <t>Demo login redirects to dashboard</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:28 pm</t>
+    <t>13/7/2026, 9:21:27 am</t>
   </si>
   <si>
     <t>TC007</t>
@@ -91,9 +91,6 @@
     <t>Dashboard visible after demo login</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:29 pm</t>
-  </si>
-  <si>
     <t>TC008</t>
   </si>
   <si>
@@ -121,7 +118,7 @@
     <t>Dashboard Total Scans card</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:32 pm</t>
+    <t>13/7/2026, 9:21:30 am</t>
   </si>
   <si>
     <t>TC012</t>
@@ -160,6 +157,9 @@
     <t>Dashboard risk distribution section</t>
   </si>
   <si>
+    <t>13/7/2026, 9:21:31 am</t>
+  </si>
+  <si>
     <t>TC018</t>
   </si>
   <si>
@@ -184,7 +184,7 @@
     <t>Scan page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:36 pm</t>
+    <t>13/7/2026, 9:21:34 am</t>
   </si>
   <si>
     <t>TC022</t>
@@ -217,7 +217,7 @@
     <t>Symptom scan returns AI results</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:50 pm</t>
+    <t>13/7/2026, 9:21:48 am</t>
   </si>
   <si>
     <t>TC027</t>
@@ -256,7 +256,7 @@
     <t>Mode B biomarker mode works</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:55 pm</t>
+    <t>13/7/2026, 9:21:53 am</t>
   </si>
   <si>
     <t>TC033</t>
@@ -265,7 +265,7 @@
     <t>Cases list page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:58 pm</t>
+    <t>13/7/2026, 9:21:57 am</t>
   </si>
   <si>
     <t>TC034</t>
@@ -298,16 +298,13 @@
     <t>Cases shows risk level pills</t>
   </si>
   <si>
-    <t>12/7/2026, 10:01:59 pm</t>
-  </si>
-  <si>
     <t>TC039</t>
   </si>
   <si>
     <t>Case detail page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:02 pm</t>
+    <t>13/7/2026, 9:22:00 am</t>
   </si>
   <si>
     <t>TC040</t>
@@ -334,7 +331,7 @@
     <t>Patients page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:06 pm</t>
+    <t>13/7/2026, 9:22:04 am</t>
   </si>
   <si>
     <t>TC044</t>
@@ -355,7 +352,7 @@
     <t>Patient selection shows timeline</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:09 pm</t>
+    <t>13/7/2026, 9:22:07 am</t>
   </si>
   <si>
     <t>TC047</t>
@@ -376,7 +373,7 @@
     <t>Alerts page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:12 pm</t>
+    <t>13/7/2026, 9:22:10 am</t>
   </si>
   <si>
     <t>TC050</t>
@@ -403,7 +400,7 @@
     <t>Bell icon links to alerts</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:16 pm</t>
+    <t>13/7/2026, 9:22:14 am</t>
   </si>
   <si>
     <t>TC054</t>
@@ -412,7 +409,7 @@
     <t>Sensors page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:20 pm</t>
+    <t>13/7/2026, 9:22:17 am</t>
   </si>
   <si>
     <t>TC055</t>
@@ -469,7 +466,7 @@
     <t>Simulator page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:23 pm</t>
+    <t>13/7/2026, 9:22:21 am</t>
   </si>
   <si>
     <t>TC064</t>
@@ -514,7 +511,7 @@
     <t>Simulator run scan generates live signal</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:33 pm</t>
+    <t>13/7/2026, 9:22:31 am</t>
   </si>
   <si>
     <t>TC071</t>
@@ -523,7 +520,7 @@
     <t>Pathogen library loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:37 pm</t>
+    <t>13/7/2026, 9:22:34 am</t>
   </si>
   <si>
     <t>TC072</t>
@@ -556,7 +553,7 @@
     <t>Pathogen detail page loads on click</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:40 pm</t>
+    <t>13/7/2026, 9:22:37 am</t>
   </si>
   <si>
     <t>TC077</t>
@@ -565,7 +562,7 @@
     <t>Compare page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:43 pm</t>
+    <t>13/7/2026, 9:22:40 am</t>
   </si>
   <si>
     <t>TC078</t>
@@ -592,7 +589,7 @@
     <t>Analytics page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:47 pm</t>
+    <t>13/7/2026, 9:22:44 am</t>
   </si>
   <si>
     <t>TC082</t>
@@ -625,7 +622,7 @@
     <t>History page shows scan records</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:50 pm</t>
+    <t>13/7/2026, 9:22:47 am</t>
   </si>
   <si>
     <t>TC087</t>
@@ -640,7 +637,7 @@
     <t>Outbreaks page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:54 pm</t>
+    <t>13/7/2026, 9:22:51 am</t>
   </si>
   <si>
     <t>TC089</t>
@@ -655,7 +652,7 @@
     <t>Settings page loads</t>
   </si>
   <si>
-    <t>12/7/2026, 10:02:57 pm</t>
+    <t>13/7/2026, 9:22:54 am</t>
   </si>
   <si>
     <t>TC091</t>
@@ -682,13 +679,580 @@
     <t>Settings has Save profile button</t>
   </si>
   <si>
+    <t>TC101</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:22:57 am</t>
+  </si>
+  <si>
+    <t>TC102</t>
+  </si>
+  <si>
+    <t>Library shows MRSA</t>
+  </si>
+  <si>
+    <t>TC103</t>
+  </si>
+  <si>
+    <t>Library shows Klebsiella pneumoniae</t>
+  </si>
+  <si>
+    <t>TC104</t>
+  </si>
+  <si>
+    <t>Library shows E. coli</t>
+  </si>
+  <si>
+    <t>TC105</t>
+  </si>
+  <si>
+    <t>Library shows Acinetobacter baumannii</t>
+  </si>
+  <si>
+    <t>TC106</t>
+  </si>
+  <si>
+    <t>Library shows Staphylococcus aureus</t>
+  </si>
+  <si>
+    <t>TC107</t>
+  </si>
+  <si>
+    <t>Library shows Streptococcus pneumoniae</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>TC108</t>
+  </si>
+  <si>
+    <t>Library shows Enterococcus faecalis</t>
+  </si>
+  <si>
+    <t>TC109</t>
+  </si>
+  <si>
+    <t>Library shows Candida albicans</t>
+  </si>
+  <si>
+    <t>TC110</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #1 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:03 am</t>
+  </si>
+  <si>
+    <t>TC111</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #2 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:06 am</t>
+  </si>
+  <si>
+    <t>TC112</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #3 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:09 am</t>
+  </si>
+  <si>
+    <t>TC113</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #4 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:11 am</t>
+  </si>
+  <si>
+    <t>TC114</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #5 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:14 am</t>
+  </si>
+  <si>
+    <t>TC115</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #6 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:16 am</t>
+  </si>
+  <si>
+    <t>TC116</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #7 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:19 am</t>
+  </si>
+  <si>
+    <t>TC117</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #8 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:22 am</t>
+  </si>
+  <si>
+    <t>TC118</t>
+  </si>
+  <si>
+    <t>Compare Pseudomonas aeruginosa vs MRSA shows QS</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:28 am</t>
+  </si>
+  <si>
+    <t>TC119</t>
+  </si>
+  <si>
+    <t>Compare Pseudomonas aeruginosa vs MRSA shows treatment</t>
+  </si>
+  <si>
+    <t>TC120</t>
+  </si>
+  <si>
+    <t>Compare Klebsiella pneumoniae vs E. coli shows QS</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:33 am</t>
+  </si>
+  <si>
+    <t>TC121</t>
+  </si>
+  <si>
+    <t>Compare Klebsiella pneumoniae vs E. coli shows treatment</t>
+  </si>
+  <si>
+    <t>TC122</t>
+  </si>
+  <si>
+    <t>Compare Acinetobacter baumannii vs Staphylococcus aureus shows QS</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:38 am</t>
+  </si>
+  <si>
+    <t>TC123</t>
+  </si>
+  <si>
+    <t>Compare Acinetobacter baumannii vs Staphylococcus aureus shows treatment</t>
+  </si>
+  <si>
+    <t>TC124</t>
+  </si>
+  <si>
+    <t>Compare Streptococcus pneumoniae vs Enterococcus faecalis shows QS</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:43 am</t>
+  </si>
+  <si>
+    <t>TC125</t>
+  </si>
+  <si>
+    <t>Compare Streptococcus pneumoniae vs Enterococcus faecalis shows treatment</t>
+  </si>
+  <si>
+    <t>TC126</t>
+  </si>
+  <si>
+    <t>Simulator DPV platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:47 am</t>
+  </si>
+  <si>
+    <t>TC127</t>
+  </si>
+  <si>
+    <t>Simulator Piezoelectric platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:48 am</t>
+  </si>
+  <si>
+    <t>TC128</t>
+  </si>
+  <si>
+    <t>Simulator FRET platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:49 am</t>
+  </si>
+  <si>
+    <t>TC129</t>
+  </si>
+  <si>
+    <t>Simulator Lateral Flow platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:50 am</t>
+  </si>
+  <si>
+    <t>TC130</t>
+  </si>
+  <si>
+    <t>Simulator MIP platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:51 am</t>
+  </si>
+  <si>
+    <t>TC131</t>
+  </si>
+  <si>
+    <t>Route /dashboard loads (Dashboard)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:55 am</t>
+  </si>
+  <si>
+    <t>TC132</t>
+  </si>
+  <si>
+    <t>Route /scan loads (Scan)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:23:59 am</t>
+  </si>
+  <si>
+    <t>TC133</t>
+  </si>
+  <si>
+    <t>Route /cases loads (Case)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:03 am</t>
+  </si>
+  <si>
+    <t>TC134</t>
+  </si>
+  <si>
+    <t>Route /patients loads (Patient)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:06 am</t>
+  </si>
+  <si>
+    <t>TC135</t>
+  </si>
+  <si>
+    <t>Route /alerts loads (Alert)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:10 am</t>
+  </si>
+  <si>
+    <t>TC136</t>
+  </si>
+  <si>
+    <t>Route /sensors loads (Sensor)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:13 am</t>
+  </si>
+  <si>
+    <t>TC137</t>
+  </si>
+  <si>
+    <t>Route /simulator loads (Simulator)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:17 am</t>
+  </si>
+  <si>
+    <t>TC138</t>
+  </si>
+  <si>
+    <t>Route /library loads (Pathogen)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:20 am</t>
+  </si>
+  <si>
+    <t>TC139</t>
+  </si>
+  <si>
+    <t>Route /compare loads (Compare)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:23 am</t>
+  </si>
+  <si>
+    <t>TC140</t>
+  </si>
+  <si>
+    <t>Route /analytics loads (Analytics)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:27 am</t>
+  </si>
+  <si>
+    <t>TC141</t>
+  </si>
+  <si>
+    <t>Route /history loads (History)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:30 am</t>
+  </si>
+  <si>
+    <t>TC142</t>
+  </si>
+  <si>
+    <t>Route /outbreaks loads (Outbreak)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:34 am</t>
+  </si>
+  <si>
+    <t>TC143</t>
+  </si>
+  <si>
+    <t>Route /settings loads (Settings)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:37 am</t>
+  </si>
+  <si>
+    <t>TC144</t>
+  </si>
+  <si>
+    <t>Forgot-password valid id shows reset info</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:42 am</t>
+  </si>
+  <si>
+    <t>TC145</t>
+  </si>
+  <si>
+    <t>Forgot-password invalid id shows error</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:47 am</t>
+  </si>
+  <si>
+    <t>TC146</t>
+  </si>
+  <si>
+    <t>Cases search filters to empty for gibberish query</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:52 am</t>
+  </si>
+  <si>
+    <t>TC147</t>
+  </si>
+  <si>
+    <t>Cases status filter controls present</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:55 am</t>
+  </si>
+  <si>
+    <t>TC148</t>
+  </si>
+  <si>
+    <t>History has risk/patient filter dropdown</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:24:59 am</t>
+  </si>
+  <si>
+    <t>TC149</t>
+  </si>
+  <si>
+    <t>Alerts has mark-read control(s)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:02 am</t>
+  </si>
+  <si>
+    <t>TC150</t>
+  </si>
+  <si>
+    <t>Theme toggle changes html class</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:06 am</t>
+  </si>
+  <si>
+    <t>TC151</t>
+  </si>
+  <si>
+    <t>Case #1 has PDF/Download</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:13 am</t>
+  </si>
+  <si>
+    <t>TC152</t>
+  </si>
+  <si>
+    <t>Case #1 shows clinical notes</t>
+  </si>
+  <si>
+    <t>TC153</t>
+  </si>
+  <si>
+    <t>Case #1 has Email/Print</t>
+  </si>
+  <si>
+    <t>TC154</t>
+  </si>
+  <si>
+    <t>Case #2 has PDF/Download</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:16 am</t>
+  </si>
+  <si>
+    <t>TC155</t>
+  </si>
+  <si>
+    <t>Case #2 shows clinical notes</t>
+  </si>
+  <si>
+    <t>TC156</t>
+  </si>
+  <si>
+    <t>Case #2 has Email/Print</t>
+  </si>
+  <si>
+    <t>TC157</t>
+  </si>
+  <si>
+    <t>Case #3 has PDF/Download</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:19 am</t>
+  </si>
+  <si>
+    <t>TC158</t>
+  </si>
+  <si>
+    <t>Case #3 shows clinical notes</t>
+  </si>
+  <si>
+    <t>TC159</t>
+  </si>
+  <si>
+    <t>Case #3 has Email/Print</t>
+  </si>
+  <si>
+    <t>TC160</t>
+  </si>
+  <si>
+    <t>Patient row #1 timeline loads</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:24 am</t>
+  </si>
+  <si>
+    <t>TC161</t>
+  </si>
+  <si>
+    <t>Patient row #2 timeline loads</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:26 am</t>
+  </si>
+  <si>
+    <t>TC162</t>
+  </si>
+  <si>
+    <t>Patient row #3 timeline loads</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:27 am</t>
+  </si>
+  <si>
+    <t>TC163</t>
+  </si>
+  <si>
+    <t>Nonexistent case id handled gracefully</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:30 am</t>
+  </si>
+  <si>
+    <t>TC164</t>
+  </si>
+  <si>
+    <t>Nonexistent patient id handled gracefully</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:32 am</t>
+  </si>
+  <si>
+    <t>TC165</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /dashboard redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:36 am</t>
+  </si>
+  <si>
+    <t>TC166</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /cases redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:39 am</t>
+  </si>
+  <si>
+    <t>TC167</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /patients redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:42 am</t>
+  </si>
+  <si>
+    <t>TC168</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /alerts redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:46 am</t>
+  </si>
+  <si>
+    <t>TC169</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /settings redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 9:25:49 am</t>
+  </si>
+  <si>
     <t>TC095</t>
   </si>
   <si>
     <t>Backend health API healthy</t>
   </si>
   <si>
-    <t>12/7/2026, 10:03:00 pm</t>
+    <t>13/7/2026, 9:26:01 am</t>
   </si>
   <si>
     <t>TC096</t>
@@ -697,7 +1261,7 @@
     <t>Backend dashboard API returns stats</t>
   </si>
   <si>
-    <t>12/7/2026, 10:03:04 pm</t>
+    <t>13/7/2026, 9:26:05 am</t>
   </si>
   <si>
     <t>TC097</t>
@@ -706,7 +1270,7 @@
     <t>Backend scans API returns records</t>
   </si>
   <si>
-    <t>12/7/2026, 10:03:08 pm</t>
+    <t>13/7/2026, 9:26:09 am</t>
   </si>
   <si>
     <t>TC098</t>
@@ -715,7 +1279,7 @@
     <t>Backend patients API returns data</t>
   </si>
   <si>
-    <t>12/7/2026, 10:03:12 pm</t>
+    <t>13/7/2026, 9:26:13 am</t>
   </si>
   <si>
     <t>TC099</t>
@@ -724,7 +1288,7 @@
     <t>Backend outbreaks API returns data</t>
   </si>
   <si>
-    <t>12/7/2026, 10:03:14 pm</t>
+    <t>13/7/2026, 9:26:15 am</t>
   </si>
   <si>
     <t>TC100</t>
@@ -733,19 +1297,19 @@
     <t>Sign out redirects to login</t>
   </si>
   <si>
-    <t>12/7/2026, 10:03:21 pm</t>
+    <t>13/7/2026, 9:26:22 am</t>
   </si>
   <si>
     <t>SUMMARY</t>
   </si>
   <si>
-    <t>Total:100</t>
-  </si>
-  <si>
-    <t>Pass:100</t>
-  </si>
-  <si>
-    <t>Fail:0</t>
+    <t>Total:169</t>
+  </si>
+  <si>
+    <t>Pass:166</t>
+  </si>
+  <si>
+    <t>Fail:3</t>
   </si>
   <si>
     <t>Skip:0</t>
@@ -771,7 +1335,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -786,6 +1350,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -806,12 +1375,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1151,7 +1722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E172"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1294,16 +1865,16 @@
         <v>8</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="C9" s="3" t="s">
         <v>7</v>
       </c>
@@ -1311,33 +1882,33 @@
         <v>8</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="E10" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="C11" s="3" t="s">
         <v>7</v>
       </c>
@@ -1345,33 +1916,33 @@
         <v>8</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="C13" s="3" t="s">
         <v>7</v>
       </c>
@@ -1379,16 +1950,16 @@
         <v>8</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="C14" s="3" t="s">
         <v>7</v>
       </c>
@@ -1396,16 +1967,16 @@
         <v>8</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="C15" s="3" t="s">
         <v>7</v>
       </c>
@@ -1413,16 +1984,16 @@
         <v>8</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="C16" s="3" t="s">
         <v>7</v>
       </c>
@@ -1430,16 +2001,16 @@
         <v>8</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="C17" s="3" t="s">
         <v>7</v>
       </c>
@@ -1447,24 +2018,24 @@
         <v>8</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1481,7 +2052,7 @@
         <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1498,7 +2069,7 @@
         <v>8</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1515,7 +2086,7 @@
         <v>8</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1821,33 +2392,33 @@
         <v>8</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="41" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>100</v>
-      </c>
       <c r="C41" s="3" t="s">
         <v>7</v>
       </c>
@@ -1855,16 +2426,16 @@
         <v>8</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="42" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>102</v>
-      </c>
       <c r="C42" s="3" t="s">
         <v>7</v>
       </c>
@@ -1872,16 +2443,16 @@
         <v>8</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="C43" s="3" t="s">
         <v>7</v>
       </c>
@@ -1889,33 +2460,33 @@
         <v>8</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="C44" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="C45" s="3" t="s">
         <v>7</v>
       </c>
@@ -1923,16 +2494,16 @@
         <v>8</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="46" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="C46" s="3" t="s">
         <v>7</v>
       </c>
@@ -1940,33 +2511,33 @@
         <v>8</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="47" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="C47" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="48" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>116</v>
-      </c>
       <c r="C48" s="3" t="s">
         <v>7</v>
       </c>
@@ -1974,16 +2545,16 @@
         <v>8</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>118</v>
-      </c>
       <c r="C49" s="3" t="s">
         <v>7</v>
       </c>
@@ -1991,33 +2562,33 @@
         <v>8</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="50" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="C50" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="51" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>123</v>
-      </c>
       <c r="C51" s="3" t="s">
         <v>7</v>
       </c>
@@ -2025,16 +2596,16 @@
         <v>8</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="52" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="C52" s="3" t="s">
         <v>7</v>
       </c>
@@ -2042,16 +2613,16 @@
         <v>8</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="53" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>127</v>
-      </c>
       <c r="C53" s="3" t="s">
         <v>7</v>
       </c>
@@ -2059,50 +2630,50 @@
         <v>8</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="54" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="C54" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="55" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="C55" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="56" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>135</v>
-      </c>
       <c r="C56" s="3" t="s">
         <v>7</v>
       </c>
@@ -2110,16 +2681,16 @@
         <v>8</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>137</v>
-      </c>
       <c r="C57" s="3" t="s">
         <v>7</v>
       </c>
@@ -2127,16 +2698,16 @@
         <v>8</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="58" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>139</v>
-      </c>
       <c r="C58" s="3" t="s">
         <v>7</v>
       </c>
@@ -2144,16 +2715,16 @@
         <v>8</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="59" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B59" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B59" s="2" t="s">
-        <v>141</v>
-      </c>
       <c r="C59" s="3" t="s">
         <v>7</v>
       </c>
@@ -2161,16 +2732,16 @@
         <v>8</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>143</v>
-      </c>
       <c r="C60" s="3" t="s">
         <v>7</v>
       </c>
@@ -2178,16 +2749,16 @@
         <v>8</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="61" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B61" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B61" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="C61" s="3" t="s">
         <v>7</v>
       </c>
@@ -2195,16 +2766,16 @@
         <v>8</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B62" s="2" t="s">
-        <v>147</v>
-      </c>
       <c r="C62" s="3" t="s">
         <v>7</v>
       </c>
@@ -2212,16 +2783,16 @@
         <v>8</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B63" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="C63" s="3" t="s">
         <v>7</v>
       </c>
@@ -2229,33 +2800,33 @@
         <v>8</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B64" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="C64" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="65" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B65" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B65" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="C65" s="3" t="s">
         <v>7</v>
       </c>
@@ -2263,16 +2834,16 @@
         <v>8</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B66" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="C66" s="3" t="s">
         <v>7</v>
       </c>
@@ -2280,16 +2851,16 @@
         <v>8</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B67" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B67" s="2" t="s">
-        <v>158</v>
-      </c>
       <c r="C67" s="3" t="s">
         <v>7</v>
       </c>
@@ -2297,16 +2868,16 @@
         <v>8</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B68" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B68" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="C68" s="3" t="s">
         <v>7</v>
       </c>
@@ -2314,16 +2885,16 @@
         <v>8</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B69" s="2" t="s">
-        <v>162</v>
-      </c>
       <c r="C69" s="3" t="s">
         <v>7</v>
       </c>
@@ -2331,16 +2902,16 @@
         <v>8</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B70" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B70" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="C70" s="3" t="s">
         <v>7</v>
       </c>
@@ -2348,50 +2919,50 @@
         <v>8</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B71" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="C71" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B72" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="C72" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E72" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B73" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B73" s="2" t="s">
-        <v>172</v>
-      </c>
       <c r="C73" s="3" t="s">
         <v>7</v>
       </c>
@@ -2399,16 +2970,16 @@
         <v>8</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B74" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="C74" s="3" t="s">
         <v>7</v>
       </c>
@@ -2416,16 +2987,16 @@
         <v>8</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B75" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B75" s="2" t="s">
-        <v>176</v>
-      </c>
       <c r="C75" s="3" t="s">
         <v>7</v>
       </c>
@@ -2433,16 +3004,16 @@
         <v>8</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B76" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B76" s="2" t="s">
-        <v>178</v>
-      </c>
       <c r="C76" s="3" t="s">
         <v>7</v>
       </c>
@@ -2450,50 +3021,50 @@
         <v>8</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="C77" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E77" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B78" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="C78" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E78" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B79" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B79" s="2" t="s">
-        <v>186</v>
-      </c>
       <c r="C79" s="3" t="s">
         <v>7</v>
       </c>
@@ -2501,16 +3072,16 @@
         <v>8</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="80" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="B80" s="2" t="s">
-        <v>188</v>
-      </c>
       <c r="C80" s="3" t="s">
         <v>7</v>
       </c>
@@ -2518,16 +3089,16 @@
         <v>8</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B81" s="2" t="s">
-        <v>190</v>
-      </c>
       <c r="C81" s="3" t="s">
         <v>7</v>
       </c>
@@ -2535,33 +3106,33 @@
         <v>8</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B82" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="C82" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E82" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="C82" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="83" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B83" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="B83" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="C83" s="3" t="s">
         <v>7</v>
       </c>
@@ -2569,16 +3140,16 @@
         <v>8</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="84" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B84" s="2" t="s">
-        <v>197</v>
-      </c>
       <c r="C84" s="3" t="s">
         <v>7</v>
       </c>
@@ -2586,16 +3157,16 @@
         <v>8</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="85" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B85" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>199</v>
-      </c>
       <c r="C85" s="3" t="s">
         <v>7</v>
       </c>
@@ -2603,16 +3174,16 @@
         <v>8</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="86" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B86" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B86" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="C86" s="3" t="s">
         <v>7</v>
       </c>
@@ -2620,33 +3191,33 @@
         <v>8</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="87" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B87" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="C87" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E87" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="C87" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="88" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B88" s="2" t="s">
-        <v>206</v>
-      </c>
       <c r="C88" s="3" t="s">
         <v>7</v>
       </c>
@@ -2654,33 +3225,33 @@
         <v>8</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="89" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B89" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="C89" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E89" s="2" t="s">
         <v>208</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="90" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B90" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B90" s="2" t="s">
-        <v>211</v>
-      </c>
       <c r="C90" s="3" t="s">
         <v>7</v>
       </c>
@@ -2688,33 +3259,33 @@
         <v>8</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="91" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B91" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B91" s="2" t="s">
+      <c r="C91" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E91" s="2" t="s">
         <v>213</v>
-      </c>
-      <c r="C91" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="92" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B92" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B92" s="2" t="s">
-        <v>216</v>
-      </c>
       <c r="C92" s="3" t="s">
         <v>7</v>
       </c>
@@ -2722,16 +3293,16 @@
         <v>8</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="93" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B93" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B93" s="2" t="s">
-        <v>218</v>
-      </c>
       <c r="C93" s="3" t="s">
         <v>7</v>
       </c>
@@ -2739,16 +3310,16 @@
         <v>8</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="94" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B94" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B94" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="C94" s="3" t="s">
         <v>7</v>
       </c>
@@ -2756,16 +3327,16 @@
         <v>8</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="95" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B95" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="B95" s="2" t="s">
-        <v>222</v>
-      </c>
       <c r="C95" s="3" t="s">
         <v>7</v>
       </c>
@@ -2773,32 +3344,32 @@
         <v>8</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="96" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E96" s="2" t="s">
         <v>223</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E96" s="2" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="97" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C97" s="3" t="s">
         <v>7</v>
@@ -2807,15 +3378,15 @@
         <v>8</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
     </row>
     <row r="98" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C98" s="3" t="s">
         <v>7</v>
@@ -2824,15 +3395,15 @@
         <v>8</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
     </row>
     <row r="99" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C99" s="3" t="s">
         <v>7</v>
@@ -2841,15 +3412,15 @@
         <v>8</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
     </row>
     <row r="100" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>7</v>
@@ -2858,15 +3429,15 @@
         <v>8</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="101" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>7</v>
@@ -2875,24 +3446,1197 @@
         <v>8</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>240</v>
+        <v>223</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E102" s="4" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="103" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C103" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="D103" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E103" s="4" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C104" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E104" s="4" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B103" s="4" t="s">
+      <c r="B105" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C103" s="4" t="s">
+      <c r="C105" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E105" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="D103" s="4" t="s">
+    </row>
+    <row r="106" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="E103" s="4" t="s">
+      <c r="B106" s="2" t="s">
         <v>245</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C137" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C151" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C153" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D153" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A154" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="C154" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="C155" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A156" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C156" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="C157" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E158" s="2" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="C159" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="C160" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E160" s="2" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="C161" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E161" s="2" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="C162" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E162" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="C163" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E163" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="C164" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E164" s="2" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="C165" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E165" s="2" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="C166" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="C167" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="B168" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="C168" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E168" s="2" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A169" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="C169" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E169" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A170" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B170" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="C170" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D170" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E170" s="2" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="B172" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="C172" s="6" t="s">
+        <v>431</v>
+      </c>
+      <c r="D172" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="E172" s="6" t="s">
+        <v>433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: send full pathogen data to compare/ask endpoints, not backend ids
</commit_message>
<xml_diff>
--- a/tests/reports/selenium-report.xlsx
+++ b/tests/reports/selenium-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="518">
   <si>
     <t>Test ID</t>
   </si>
@@ -40,7 +40,7 @@
     <t/>
   </si>
   <si>
-    <t>13/7/2026, 9:21:09 am</t>
+    <t>13/7/2026, 10:24:30 am</t>
   </si>
   <si>
     <t>TC002</t>
@@ -55,7 +55,7 @@
     <t>Login page shows ChemoSense branding</t>
   </si>
   <si>
-    <t>13/7/2026, 9:21:13 am</t>
+    <t>13/7/2026, 10:24:34 am</t>
   </si>
   <si>
     <t>TC004</t>
@@ -73,7 +73,7 @@
     <t>Invalid login shows error message</t>
   </si>
   <si>
-    <t>13/7/2026, 9:21:16 am</t>
+    <t>13/7/2026, 10:24:37 am</t>
   </si>
   <si>
     <t>TC006</t>
@@ -82,7 +82,7 @@
     <t>Demo login redirects to dashboard</t>
   </si>
   <si>
-    <t>13/7/2026, 9:21:27 am</t>
+    <t>13/7/2026, 10:24:48 am</t>
   </si>
   <si>
     <t>TC007</t>
@@ -118,7 +118,7 @@
     <t>Dashboard Total Scans card</t>
   </si>
   <si>
-    <t>13/7/2026, 9:21:30 am</t>
+    <t>13/7/2026, 10:24:52 am</t>
   </si>
   <si>
     <t>TC012</t>
@@ -157,9 +157,6 @@
     <t>Dashboard risk distribution section</t>
   </si>
   <si>
-    <t>13/7/2026, 9:21:31 am</t>
-  </si>
-  <si>
     <t>TC018</t>
   </si>
   <si>
@@ -184,7 +181,7 @@
     <t>Scan page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:21:34 am</t>
+    <t>13/7/2026, 10:24:55 am</t>
   </si>
   <si>
     <t>TC022</t>
@@ -211,13 +208,16 @@
     <t>Scan textarea accepts input</t>
   </si>
   <si>
+    <t>13/7/2026, 10:24:56 am</t>
+  </si>
+  <si>
     <t>TC026</t>
   </si>
   <si>
     <t>Symptom scan returns AI results</t>
   </si>
   <si>
-    <t>13/7/2026, 9:21:48 am</t>
+    <t>13/7/2026, 10:25:09 am</t>
   </si>
   <si>
     <t>TC027</t>
@@ -256,7 +256,7 @@
     <t>Mode B biomarker mode works</t>
   </si>
   <si>
-    <t>13/7/2026, 9:21:53 am</t>
+    <t>13/7/2026, 10:25:14 am</t>
   </si>
   <si>
     <t>TC033</t>
@@ -265,7 +265,7 @@
     <t>Cases list page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:21:57 am</t>
+    <t>13/7/2026, 10:25:18 am</t>
   </si>
   <si>
     <t>TC034</t>
@@ -304,7 +304,7 @@
     <t>Case detail page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:00 am</t>
+    <t>13/7/2026, 10:25:22 am</t>
   </si>
   <si>
     <t>TC040</t>
@@ -331,7 +331,7 @@
     <t>Patients page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:04 am</t>
+    <t>13/7/2026, 10:25:25 am</t>
   </si>
   <si>
     <t>TC044</t>
@@ -352,7 +352,7 @@
     <t>Patient selection shows timeline</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:07 am</t>
+    <t>13/7/2026, 10:25:29 am</t>
   </si>
   <si>
     <t>TC047</t>
@@ -373,7 +373,7 @@
     <t>Alerts page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:10 am</t>
+    <t>13/7/2026, 10:25:32 am</t>
   </si>
   <si>
     <t>TC050</t>
@@ -400,7 +400,7 @@
     <t>Bell icon links to alerts</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:14 am</t>
+    <t>13/7/2026, 10:25:36 am</t>
   </si>
   <si>
     <t>TC054</t>
@@ -409,7 +409,7 @@
     <t>Sensors page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:17 am</t>
+    <t>13/7/2026, 10:25:42 am</t>
   </si>
   <si>
     <t>TC055</t>
@@ -466,7 +466,7 @@
     <t>Simulator page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:21 am</t>
+    <t>13/7/2026, 10:25:45 am</t>
   </si>
   <si>
     <t>TC064</t>
@@ -475,6 +475,9 @@
     <t>DPV Colorimetric platform visible</t>
   </si>
   <si>
+    <t>13/7/2026, 10:25:46 am</t>
+  </si>
+  <si>
     <t>TC065</t>
   </si>
   <si>
@@ -511,7 +514,7 @@
     <t>Simulator run scan generates live signal</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:31 am</t>
+    <t>13/7/2026, 10:25:56 am</t>
   </si>
   <si>
     <t>TC071</t>
@@ -520,7 +523,7 @@
     <t>Pathogen library loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:34 am</t>
+    <t>13/7/2026, 10:25:59 am</t>
   </si>
   <si>
     <t>TC072</t>
@@ -553,7 +556,7 @@
     <t>Pathogen detail page loads on click</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:37 am</t>
+    <t>13/7/2026, 10:26:02 am</t>
   </si>
   <si>
     <t>TC077</t>
@@ -562,7 +565,7 @@
     <t>Compare page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:40 am</t>
+    <t>13/7/2026, 10:26:07 am</t>
   </si>
   <si>
     <t>TC078</t>
@@ -589,7 +592,7 @@
     <t>Analytics page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:44 am</t>
+    <t>13/7/2026, 10:26:10 am</t>
   </si>
   <si>
     <t>TC082</t>
@@ -622,7 +625,7 @@
     <t>History page shows scan records</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:47 am</t>
+    <t>13/7/2026, 10:26:14 am</t>
   </si>
   <si>
     <t>TC087</t>
@@ -637,7 +640,7 @@
     <t>Outbreaks page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:51 am</t>
+    <t>13/7/2026, 10:26:18 am</t>
   </si>
   <si>
     <t>TC089</t>
@@ -652,7 +655,7 @@
     <t>Settings page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:54 am</t>
+    <t>13/7/2026, 10:26:21 am</t>
   </si>
   <si>
     <t>TC091</t>
@@ -682,27 +685,27 @@
     <t>TC101</t>
   </si>
   <si>
-    <t>13/7/2026, 9:22:57 am</t>
+    <t>13/7/2026, 10:26:25 am</t>
   </si>
   <si>
     <t>TC102</t>
   </si>
   <si>
-    <t>Library shows MRSA</t>
+    <t>Library shows Staphylococcus aureus</t>
   </si>
   <si>
     <t>TC103</t>
   </si>
   <si>
+    <t>Library shows Escherichia coli</t>
+  </si>
+  <si>
+    <t>TC104</t>
+  </si>
+  <si>
     <t>Library shows Klebsiella pneumoniae</t>
   </si>
   <si>
-    <t>TC104</t>
-  </si>
-  <si>
-    <t>Library shows E. coli</t>
-  </si>
-  <si>
     <t>TC105</t>
   </si>
   <si>
@@ -712,538 +715,788 @@
     <t>TC106</t>
   </si>
   <si>
-    <t>Library shows Staphylococcus aureus</t>
+    <t>Library shows Enterococcus faecium</t>
   </si>
   <si>
     <t>TC107</t>
   </si>
   <si>
-    <t>Library shows Streptococcus pneumoniae</t>
+    <t>Library shows Mycobacterium tuberculosis</t>
+  </si>
+  <si>
+    <t>TC108</t>
+  </si>
+  <si>
+    <t>Library shows Vibrio cholerae</t>
+  </si>
+  <si>
+    <t>TC109</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #1 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:26:31 am</t>
+  </si>
+  <si>
+    <t>TC110</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #2 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:26:33 am</t>
+  </si>
+  <si>
+    <t>TC111</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #3 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:26:36 am</t>
+  </si>
+  <si>
+    <t>TC112</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #4 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:26:39 am</t>
+  </si>
+  <si>
+    <t>TC113</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #5 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:26:41 am</t>
+  </si>
+  <si>
+    <t>TC114</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #6 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:26:44 am</t>
+  </si>
+  <si>
+    <t>TC115</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #7 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:26:46 am</t>
+  </si>
+  <si>
+    <t>TC116</t>
+  </si>
+  <si>
+    <t>Pathogen detail card #8 renders</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:26:49 am</t>
+  </si>
+  <si>
+    <t>TC117</t>
+  </si>
+  <si>
+    <t>Compare Pseudomonas aeruginosa vs Staphylococcus aureus shows QS</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:26:55 am</t>
+  </si>
+  <si>
+    <t>TC118</t>
+  </si>
+  <si>
+    <t>Compare Pseudomonas aeruginosa vs Staphylococcus aureus shows treatment</t>
+  </si>
+  <si>
+    <t>TC119</t>
+  </si>
+  <si>
+    <t>Compare Klebsiella pneumoniae vs Escherichia coli shows QS</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:04 am</t>
+  </si>
+  <si>
+    <t>TC120</t>
+  </si>
+  <si>
+    <t>Compare Klebsiella pneumoniae vs Escherichia coli shows treatment</t>
+  </si>
+  <si>
+    <t>TC121</t>
+  </si>
+  <si>
+    <t>Compare Acinetobacter baumannii vs Enterococcus faecium shows QS</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:13 am</t>
+  </si>
+  <si>
+    <t>TC122</t>
+  </si>
+  <si>
+    <t>Compare Acinetobacter baumannii vs Enterococcus faecium shows treatment</t>
+  </si>
+  <si>
+    <t>TC123</t>
+  </si>
+  <si>
+    <t>Compare Mycobacterium tuberculosis vs Vibrio cholerae shows QS</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:19 am</t>
+  </si>
+  <si>
+    <t>TC124</t>
+  </si>
+  <si>
+    <t>Compare Mycobacterium tuberculosis vs Vibrio cholerae shows treatment</t>
+  </si>
+  <si>
+    <t>TC125</t>
+  </si>
+  <si>
+    <t>Simulator DPV platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:24 am</t>
+  </si>
+  <si>
+    <t>TC126</t>
+  </si>
+  <si>
+    <t>Simulator Piezoelectric platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:25 am</t>
+  </si>
+  <si>
+    <t>TC127</t>
+  </si>
+  <si>
+    <t>Simulator FRET platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:26 am</t>
+  </si>
+  <si>
+    <t>TC128</t>
+  </si>
+  <si>
+    <t>Simulator Lateral Flow platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:27 am</t>
+  </si>
+  <si>
+    <t>TC129</t>
+  </si>
+  <si>
+    <t>Simulator MIP platform selectable, shows LOD</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:28 am</t>
+  </si>
+  <si>
+    <t>TC130</t>
+  </si>
+  <si>
+    <t>Route /dashboard loads (Dashboard)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:32 am</t>
+  </si>
+  <si>
+    <t>TC131</t>
+  </si>
+  <si>
+    <t>Route /scan loads (Scan)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:38 am</t>
+  </si>
+  <si>
+    <t>TC132</t>
+  </si>
+  <si>
+    <t>Route /cases loads (Case)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:42 am</t>
+  </si>
+  <si>
+    <t>TC133</t>
+  </si>
+  <si>
+    <t>Route /patients loads (Patient)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:45 am</t>
+  </si>
+  <si>
+    <t>TC134</t>
+  </si>
+  <si>
+    <t>Route /alerts loads (Alert)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:49 am</t>
+  </si>
+  <si>
+    <t>TC135</t>
+  </si>
+  <si>
+    <t>Route /sensors loads (Sensor)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:56 am</t>
+  </si>
+  <si>
+    <t>TC136</t>
+  </si>
+  <si>
+    <t>Route /simulator loads (Simulator)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:27:59 am</t>
+  </si>
+  <si>
+    <t>TC137</t>
+  </si>
+  <si>
+    <t>Route /library loads (Pathogen)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:03 am</t>
+  </si>
+  <si>
+    <t>TC138</t>
+  </si>
+  <si>
+    <t>Route /compare loads (Compare)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:06 am</t>
+  </si>
+  <si>
+    <t>TC139</t>
+  </si>
+  <si>
+    <t>Route /analytics loads (Analytics)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:10 am</t>
+  </si>
+  <si>
+    <t>TC140</t>
+  </si>
+  <si>
+    <t>Route /history loads (History)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:13 am</t>
+  </si>
+  <si>
+    <t>TC141</t>
+  </si>
+  <si>
+    <t>Route /outbreaks loads (Outbreak)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:17 am</t>
+  </si>
+  <si>
+    <t>TC142</t>
+  </si>
+  <si>
+    <t>Route /settings loads (Settings)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:22 am</t>
+  </si>
+  <si>
+    <t>TC143</t>
+  </si>
+  <si>
+    <t>Forgot-password valid id shows reset info</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:29 am</t>
+  </si>
+  <si>
+    <t>TC144</t>
+  </si>
+  <si>
+    <t>Forgot-password invalid id shows error</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:35 am</t>
+  </si>
+  <si>
+    <t>TC145</t>
+  </si>
+  <si>
+    <t>Cases search filters to empty for gibberish query</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:39 am</t>
+  </si>
+  <si>
+    <t>TC146</t>
+  </si>
+  <si>
+    <t>Cases status filter controls present</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:43 am</t>
+  </si>
+  <si>
+    <t>TC147</t>
+  </si>
+  <si>
+    <t>History has risk/patient filter dropdown</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:28:46 am</t>
+  </si>
+  <si>
+    <t>TC148</t>
+  </si>
+  <si>
+    <t>Alerts has mark-read control(s)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:04 am</t>
+  </si>
+  <si>
+    <t>TC149</t>
+  </si>
+  <si>
+    <t>Theme toggle changes html class</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:08 am</t>
+  </si>
+  <si>
+    <t>TC150</t>
+  </si>
+  <si>
+    <t>Case #1 has PDF/Download</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:16 am</t>
+  </si>
+  <si>
+    <t>TC151</t>
+  </si>
+  <si>
+    <t>Case #1 shows clinical notes</t>
+  </si>
+  <si>
+    <t>TC152</t>
+  </si>
+  <si>
+    <t>Case #1 has Email/Print</t>
+  </si>
+  <si>
+    <t>TC153</t>
+  </si>
+  <si>
+    <t>Case #2 has PDF/Download</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:19 am</t>
+  </si>
+  <si>
+    <t>TC154</t>
+  </si>
+  <si>
+    <t>Case #2 shows clinical notes</t>
+  </si>
+  <si>
+    <t>TC155</t>
+  </si>
+  <si>
+    <t>Case #2 has Email/Print</t>
+  </si>
+  <si>
+    <t>TC156</t>
+  </si>
+  <si>
+    <t>Case #3 has PDF/Download</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:22 am</t>
+  </si>
+  <si>
+    <t>TC157</t>
+  </si>
+  <si>
+    <t>Case #3 shows clinical notes</t>
+  </si>
+  <si>
+    <t>TC158</t>
+  </si>
+  <si>
+    <t>Case #3 has Email/Print</t>
+  </si>
+  <si>
+    <t>TC159</t>
+  </si>
+  <si>
+    <t>Patient row #1 timeline loads</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:27 am</t>
+  </si>
+  <si>
+    <t>TC160</t>
+  </si>
+  <si>
+    <t>Patient row #2 timeline loads</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:29 am</t>
+  </si>
+  <si>
+    <t>TC161</t>
+  </si>
+  <si>
+    <t>Patient row #3 timeline loads</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:30 am</t>
+  </si>
+  <si>
+    <t>TC162</t>
+  </si>
+  <si>
+    <t>Nonexistent case id handled gracefully</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:33 am</t>
+  </si>
+  <si>
+    <t>TC163</t>
+  </si>
+  <si>
+    <t>Nonexistent patient id handled gracefully</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:36 am</t>
+  </si>
+  <si>
+    <t>TC164</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /dashboard redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:39 am</t>
+  </si>
+  <si>
+    <t>TC165</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /cases redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:42 am</t>
+  </si>
+  <si>
+    <t>TC166</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /patients redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:46 am</t>
+  </si>
+  <si>
+    <t>TC167</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /alerts redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:49 am</t>
+  </si>
+  <si>
+    <t>TC168</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to /settings redirects to login</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:29:52 am</t>
+  </si>
+  <si>
+    <t>TC169</t>
+  </si>
+  <si>
+    <t>Register as technician reaches dashboard</t>
   </si>
   <si>
     <t>FAIL</t>
   </si>
   <si>
-    <t>TC108</t>
-  </si>
-  <si>
-    <t>Library shows Enterococcus faecalis</t>
-  </si>
-  <si>
-    <t>TC109</t>
-  </si>
-  <si>
-    <t>Library shows Candida albicans</t>
-  </si>
-  <si>
-    <t>TC110</t>
-  </si>
-  <si>
-    <t>Pathogen detail card #1 renders</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:03 am</t>
-  </si>
-  <si>
-    <t>TC111</t>
-  </si>
-  <si>
-    <t>Pathogen detail card #2 renders</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:06 am</t>
-  </si>
-  <si>
-    <t>TC112</t>
-  </si>
-  <si>
-    <t>Pathogen detail card #3 renders</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:09 am</t>
-  </si>
-  <si>
-    <t>TC113</t>
-  </si>
-  <si>
-    <t>Pathogen detail card #4 renders</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:11 am</t>
-  </si>
-  <si>
-    <t>TC114</t>
-  </si>
-  <si>
-    <t>Pathogen detail card #5 renders</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:14 am</t>
-  </si>
-  <si>
-    <t>TC115</t>
-  </si>
-  <si>
-    <t>Pathogen detail card #6 renders</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:16 am</t>
-  </si>
-  <si>
-    <t>TC116</t>
-  </si>
-  <si>
-    <t>Pathogen detail card #7 renders</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:19 am</t>
-  </si>
-  <si>
-    <t>TC117</t>
-  </si>
-  <si>
-    <t>Pathogen detail card #8 renders</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:22 am</t>
-  </si>
-  <si>
-    <t>TC118</t>
-  </si>
-  <si>
-    <t>Compare Pseudomonas aeruginosa vs MRSA shows QS</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:28 am</t>
-  </si>
-  <si>
-    <t>TC119</t>
-  </si>
-  <si>
-    <t>Compare Pseudomonas aeruginosa vs MRSA shows treatment</t>
-  </si>
-  <si>
-    <t>TC120</t>
-  </si>
-  <si>
-    <t>Compare Klebsiella pneumoniae vs E. coli shows QS</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:33 am</t>
-  </si>
-  <si>
-    <t>TC121</t>
-  </si>
-  <si>
-    <t>Compare Klebsiella pneumoniae vs E. coli shows treatment</t>
-  </si>
-  <si>
-    <t>TC122</t>
-  </si>
-  <si>
-    <t>Compare Acinetobacter baumannii vs Staphylococcus aureus shows QS</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:38 am</t>
-  </si>
-  <si>
-    <t>TC123</t>
-  </si>
-  <si>
-    <t>Compare Acinetobacter baumannii vs Staphylococcus aureus shows treatment</t>
-  </si>
-  <si>
-    <t>TC124</t>
-  </si>
-  <si>
-    <t>Compare Streptococcus pneumoniae vs Enterococcus faecalis shows QS</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:43 am</t>
-  </si>
-  <si>
-    <t>TC125</t>
-  </si>
-  <si>
-    <t>Compare Streptococcus pneumoniae vs Enterococcus faecalis shows treatment</t>
-  </si>
-  <si>
-    <t>TC126</t>
-  </si>
-  <si>
-    <t>Simulator DPV platform selectable, shows LOD</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:47 am</t>
-  </si>
-  <si>
-    <t>TC127</t>
-  </si>
-  <si>
-    <t>Simulator Piezoelectric platform selectable, shows LOD</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:48 am</t>
-  </si>
-  <si>
-    <t>TC128</t>
-  </si>
-  <si>
-    <t>Simulator FRET platform selectable, shows LOD</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:49 am</t>
-  </si>
-  <si>
-    <t>TC129</t>
-  </si>
-  <si>
-    <t>Simulator Lateral Flow platform selectable, shows LOD</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:50 am</t>
-  </si>
-  <si>
-    <t>TC130</t>
-  </si>
-  <si>
-    <t>Simulator MIP platform selectable, shows LOD</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:51 am</t>
-  </si>
-  <si>
-    <t>TC131</t>
-  </si>
-  <si>
-    <t>Route /dashboard loads (Dashboard)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:55 am</t>
-  </si>
-  <si>
-    <t>TC132</t>
-  </si>
-  <si>
-    <t>Route /scan loads (Scan)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:23:59 am</t>
-  </si>
-  <si>
-    <t>TC133</t>
-  </si>
-  <si>
-    <t>Route /cases loads (Case)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:03 am</t>
-  </si>
-  <si>
-    <t>TC134</t>
-  </si>
-  <si>
-    <t>Route /patients loads (Patient)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:06 am</t>
-  </si>
-  <si>
-    <t>TC135</t>
-  </si>
-  <si>
-    <t>Route /alerts loads (Alert)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:10 am</t>
-  </si>
-  <si>
-    <t>TC136</t>
-  </si>
-  <si>
-    <t>Route /sensors loads (Sensor)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:13 am</t>
-  </si>
-  <si>
-    <t>TC137</t>
-  </si>
-  <si>
-    <t>Route /simulator loads (Simulator)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:17 am</t>
-  </si>
-  <si>
-    <t>TC138</t>
-  </si>
-  <si>
-    <t>Route /library loads (Pathogen)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:20 am</t>
-  </si>
-  <si>
-    <t>TC139</t>
-  </si>
-  <si>
-    <t>Route /compare loads (Compare)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:23 am</t>
-  </si>
-  <si>
-    <t>TC140</t>
-  </si>
-  <si>
-    <t>Route /analytics loads (Analytics)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:27 am</t>
-  </si>
-  <si>
-    <t>TC141</t>
-  </si>
-  <si>
-    <t>Route /history loads (History)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:30 am</t>
-  </si>
-  <si>
-    <t>TC142</t>
-  </si>
-  <si>
-    <t>Route /outbreaks loads (Outbreak)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:34 am</t>
-  </si>
-  <si>
-    <t>TC143</t>
-  </si>
-  <si>
-    <t>Route /settings loads (Settings)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:37 am</t>
-  </si>
-  <si>
-    <t>TC144</t>
-  </si>
-  <si>
-    <t>Forgot-password valid id shows reset info</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:42 am</t>
-  </si>
-  <si>
-    <t>TC145</t>
-  </si>
-  <si>
-    <t>Forgot-password invalid id shows error</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:47 am</t>
-  </si>
-  <si>
-    <t>TC146</t>
-  </si>
-  <si>
-    <t>Cases search filters to empty for gibberish query</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:52 am</t>
-  </si>
-  <si>
-    <t>TC147</t>
-  </si>
-  <si>
-    <t>Cases status filter controls present</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:55 am</t>
-  </si>
-  <si>
-    <t>TC148</t>
-  </si>
-  <si>
-    <t>History has risk/patient filter dropdown</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:24:59 am</t>
-  </si>
-  <si>
-    <t>TC149</t>
-  </si>
-  <si>
-    <t>Alerts has mark-read control(s)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:02 am</t>
-  </si>
-  <si>
-    <t>TC150</t>
-  </si>
-  <si>
-    <t>Theme toggle changes html class</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:06 am</t>
-  </si>
-  <si>
-    <t>TC151</t>
-  </si>
-  <si>
-    <t>Case #1 has PDF/Download</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:13 am</t>
-  </si>
-  <si>
-    <t>TC152</t>
-  </si>
-  <si>
-    <t>Case #1 shows clinical notes</t>
-  </si>
-  <si>
-    <t>TC153</t>
-  </si>
-  <si>
-    <t>Case #1 has Email/Print</t>
-  </si>
-  <si>
-    <t>TC154</t>
-  </si>
-  <si>
-    <t>Case #2 has PDF/Download</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:16 am</t>
-  </si>
-  <si>
-    <t>TC155</t>
-  </si>
-  <si>
-    <t>Case #2 shows clinical notes</t>
-  </si>
-  <si>
-    <t>TC156</t>
-  </si>
-  <si>
-    <t>Case #2 has Email/Print</t>
-  </si>
-  <si>
-    <t>TC157</t>
-  </si>
-  <si>
-    <t>Case #3 has PDF/Download</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:19 am</t>
-  </si>
-  <si>
-    <t>TC158</t>
-  </si>
-  <si>
-    <t>Case #3 shows clinical notes</t>
-  </si>
-  <si>
-    <t>TC159</t>
-  </si>
-  <si>
-    <t>Case #3 has Email/Print</t>
-  </si>
-  <si>
-    <t>TC160</t>
-  </si>
-  <si>
-    <t>Patient row #1 timeline loads</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:24 am</t>
-  </si>
-  <si>
-    <t>TC161</t>
-  </si>
-  <si>
-    <t>Patient row #2 timeline loads</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:26 am</t>
-  </si>
-  <si>
-    <t>TC162</t>
-  </si>
-  <si>
-    <t>Patient row #3 timeline loads</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:27 am</t>
-  </si>
-  <si>
-    <t>TC163</t>
-  </si>
-  <si>
-    <t>Nonexistent case id handled gracefully</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:30 am</t>
-  </si>
-  <si>
-    <t>TC164</t>
-  </si>
-  <si>
-    <t>Nonexistent patient id handled gracefully</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:32 am</t>
-  </si>
-  <si>
-    <t>TC165</t>
-  </si>
-  <si>
-    <t>Unauthenticated access to /dashboard redirects to login</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:36 am</t>
-  </si>
-  <si>
-    <t>TC166</t>
-  </si>
-  <si>
-    <t>Unauthenticated access to /cases redirects to login</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:39 am</t>
-  </si>
-  <si>
-    <t>TC167</t>
-  </si>
-  <si>
-    <t>Unauthenticated access to /patients redirects to login</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:42 am</t>
-  </si>
-  <si>
-    <t>TC168</t>
-  </si>
-  <si>
-    <t>Unauthenticated access to /alerts redirects to login</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:46 am</t>
-  </si>
-  <si>
-    <t>TC169</t>
-  </si>
-  <si>
-    <t>Unauthenticated access to /settings redirects to login</t>
-  </si>
-  <si>
-    <t>13/7/2026, 9:25:49 am</t>
+    <t>https://chemosense-app.onrender.com/login?demo=false</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:09 am</t>
+  </si>
+  <si>
+    <t>TC170</t>
+  </si>
+  <si>
+    <t>Register as doctor reaches dashboard</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:17 am</t>
+  </si>
+  <si>
+    <t>TC171</t>
+  </si>
+  <si>
+    <t>Register as admin reaches dashboard</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:25 am</t>
+  </si>
+  <si>
+    <t>TC172</t>
+  </si>
+  <si>
+    <t>Change-password rejects wrong current password</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:39 am</t>
+  </si>
+  <si>
+    <t>TC173</t>
+  </si>
+  <si>
+    <t>Mode B biomarker search available (context: Pseudomonas aeruginosa)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:44 am</t>
+  </si>
+  <si>
+    <t>TC174</t>
+  </si>
+  <si>
+    <t>Mode B biomarker search available (context: Staphylococcus aureus)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:45 am</t>
+  </si>
+  <si>
+    <t>TC175</t>
+  </si>
+  <si>
+    <t>Mode B biomarker search available (context: Escherichia coli)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:46 am</t>
+  </si>
+  <si>
+    <t>TC176</t>
+  </si>
+  <si>
+    <t>Mode B biomarker search available (context: Klebsiella pneumoniae)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:47 am</t>
+  </si>
+  <si>
+    <t>TC177</t>
+  </si>
+  <si>
+    <t>Mode B biomarker search available (context: Acinetobacter baumannii)</t>
+  </si>
+  <si>
+    <t>TC178</t>
+  </si>
+  <si>
+    <t>Mode B biomarker search available (context: Enterococcus faecium)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:48 am</t>
+  </si>
+  <si>
+    <t>TC179</t>
+  </si>
+  <si>
+    <t>Mode B biomarker search available (context: Mycobacterium tuberculosis)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:49 am</t>
+  </si>
+  <si>
+    <t>TC180</t>
+  </si>
+  <si>
+    <t>Mode B biomarker search available (context: Vibrio cholerae)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:50 am</t>
+  </si>
+  <si>
+    <t>TC181</t>
+  </si>
+  <si>
+    <t>Analytics quick-fill button #1 clickable</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:54 am</t>
+  </si>
+  <si>
+    <t>TC182</t>
+  </si>
+  <si>
+    <t>Analytics quick-fill button #2 clickable</t>
+  </si>
+  <si>
+    <t>TC183</t>
+  </si>
+  <si>
+    <t>Analytics quick-fill button #3 clickable</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:55 am</t>
+  </si>
+  <si>
+    <t>TC184</t>
+  </si>
+  <si>
+    <t>Analytics quick-fill button #4 clickable</t>
+  </si>
+  <si>
+    <t>TC185</t>
+  </si>
+  <si>
+    <t>Outbreaks may reference Pseudomonas aeruginosa</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:30:59 am</t>
+  </si>
+  <si>
+    <t>TC186</t>
+  </si>
+  <si>
+    <t>Outbreaks may reference Staphylococcus aureus</t>
+  </si>
+  <si>
+    <t>TC187</t>
+  </si>
+  <si>
+    <t>Outbreaks page loaded (no Escherichia coli mention, acceptable)</t>
+  </si>
+  <si>
+    <t>SKIP</t>
+  </si>
+  <si>
+    <t>TC188</t>
+  </si>
+  <si>
+    <t>Outbreaks may reference Klebsiella pneumoniae</t>
+  </si>
+  <si>
+    <t>TC189</t>
+  </si>
+  <si>
+    <t>Outbreaks may reference Acinetobacter baumannii</t>
+  </si>
+  <si>
+    <t>TC190</t>
+  </si>
+  <si>
+    <t>Ward heatmap renders grid cells</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:31:02 am</t>
+  </si>
+  <si>
+    <t>TC192</t>
+  </si>
+  <si>
+    <t>Sensor add form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">element click intercepted: Element &lt;button class="h-9 px-3 text-xs rounded-md bg-primary text-primary-foreground inline-flex items-center gap-1.5"&gt;...&lt;/button&gt; is not clickable at point (1202, 42). Other element would receive the click: &lt;div class="fixed inset-0 bg-black/50 z-50 flex items-center justify-center p-4"&gt;...&lt;/div&gt;
+  (Session info: chrome=150.0.7871.49)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:31:08 am</t>
+  </si>
+  <si>
+    <t>TC193</t>
+  </si>
+  <si>
+    <t>Dashboard shows Critical risk tier</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:31:11 am</t>
+  </si>
+  <si>
+    <t>TC194</t>
+  </si>
+  <si>
+    <t>Dashboard shows High risk tier</t>
+  </si>
+  <si>
+    <t>TC195</t>
+  </si>
+  <si>
+    <t>Dashboard shows Moderate risk tier</t>
+  </si>
+  <si>
+    <t>TC196</t>
+  </si>
+  <si>
+    <t>Dashboard shows Low risk tier</t>
+  </si>
+  <si>
+    <t>TC197</t>
+  </si>
+  <si>
+    <t>Cases list shows Open status pill</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:31:15 am</t>
+  </si>
+  <si>
+    <t>TC198</t>
+  </si>
+  <si>
+    <t>Cases list shows Closed status pill</t>
+  </si>
+  <si>
+    <t>TC199</t>
+  </si>
+  <si>
+    <t>Settings profile field is editable</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:31:18 am</t>
+  </si>
+  <si>
+    <t>TC200</t>
+  </si>
+  <si>
+    <t>Sign out then demo sign-in round trip works</t>
+  </si>
+  <si>
+    <t>13/7/2026, 10:31:33 am</t>
   </si>
   <si>
     <t>TC095</t>
@@ -1252,7 +1505,7 @@
     <t>Backend health API healthy</t>
   </si>
   <si>
-    <t>13/7/2026, 9:26:01 am</t>
+    <t>13/7/2026, 10:31:35 am</t>
   </si>
   <si>
     <t>TC096</t>
@@ -1261,7 +1514,7 @@
     <t>Backend dashboard API returns stats</t>
   </si>
   <si>
-    <t>13/7/2026, 9:26:05 am</t>
+    <t>13/7/2026, 10:31:40 am</t>
   </si>
   <si>
     <t>TC097</t>
@@ -1270,7 +1523,7 @@
     <t>Backend scans API returns records</t>
   </si>
   <si>
-    <t>13/7/2026, 9:26:09 am</t>
+    <t>13/7/2026, 10:31:44 am</t>
   </si>
   <si>
     <t>TC098</t>
@@ -1279,7 +1532,7 @@
     <t>Backend patients API returns data</t>
   </si>
   <si>
-    <t>13/7/2026, 9:26:13 am</t>
+    <t>13/7/2026, 10:31:48 am</t>
   </si>
   <si>
     <t>TC099</t>
@@ -1288,7 +1541,7 @@
     <t>Backend outbreaks API returns data</t>
   </si>
   <si>
-    <t>13/7/2026, 9:26:15 am</t>
+    <t>13/7/2026, 10:31:51 am</t>
   </si>
   <si>
     <t>TC100</t>
@@ -1297,22 +1550,22 @@
     <t>Sign out redirects to login</t>
   </si>
   <si>
-    <t>13/7/2026, 9:26:22 am</t>
+    <t>13/7/2026, 10:31:58 am</t>
   </si>
   <si>
     <t>SUMMARY</t>
   </si>
   <si>
-    <t>Total:169</t>
-  </si>
-  <si>
-    <t>Pass:166</t>
-  </si>
-  <si>
-    <t>Fail:3</t>
-  </si>
-  <si>
-    <t>Skip:0</t>
+    <t>Total:199</t>
+  </si>
+  <si>
+    <t>Pass:193</t>
+  </si>
+  <si>
+    <t>Fail:4</t>
+  </si>
+  <si>
+    <t>Skip:2</t>
   </si>
 </sst>
 </file>
@@ -1335,7 +1588,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1359,6 +1612,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF1E293B"/>
       </patternFill>
     </fill>
@@ -1375,14 +1633,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1722,7 +1982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E172"/>
+  <dimension ref="A1:E202"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2035,16 +2295,16 @@
         <v>8</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="C19" s="3" t="s">
         <v>7</v>
       </c>
@@ -2052,16 +2312,16 @@
         <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="C20" s="3" t="s">
         <v>7</v>
       </c>
@@ -2069,16 +2329,16 @@
         <v>8</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="C21" s="3" t="s">
         <v>7</v>
       </c>
@@ -2086,33 +2346,33 @@
         <v>8</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="C23" s="3" t="s">
         <v>7</v>
       </c>
@@ -2120,16 +2380,16 @@
         <v>8</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="C24" s="3" t="s">
         <v>7</v>
       </c>
@@ -2137,16 +2397,16 @@
         <v>8</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="C25" s="3" t="s">
         <v>7</v>
       </c>
@@ -2154,24 +2414,24 @@
         <v>8</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2834,32 +3094,32 @@
         <v>8</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>7</v>
@@ -2868,15 +3128,15 @@
         <v>8</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>7</v>
@@ -2885,15 +3145,15 @@
         <v>8</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>7</v>
@@ -2902,15 +3162,15 @@
         <v>8</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>7</v>
@@ -2919,15 +3179,15 @@
         <v>8</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>7</v>
@@ -2936,15 +3196,15 @@
         <v>8</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>7</v>
@@ -2953,32 +3213,32 @@
         <v>8</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E73" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>7</v>
@@ -2987,15 +3247,15 @@
         <v>8</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C75" s="3" t="s">
         <v>7</v>
@@ -3004,15 +3264,15 @@
         <v>8</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C76" s="3" t="s">
         <v>7</v>
@@ -3021,15 +3281,15 @@
         <v>8</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C77" s="3" t="s">
         <v>7</v>
@@ -3038,15 +3298,15 @@
         <v>8</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>7</v>
@@ -3055,32 +3315,32 @@
         <v>8</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E79" s="2" t="s">
         <v>184</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="C79" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="80" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C80" s="3" t="s">
         <v>7</v>
@@ -3089,15 +3349,15 @@
         <v>8</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C81" s="3" t="s">
         <v>7</v>
@@ -3106,15 +3366,15 @@
         <v>8</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>7</v>
@@ -3123,32 +3383,32 @@
         <v>8</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="83" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E83" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="C83" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="84" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C84" s="3" t="s">
         <v>7</v>
@@ -3157,15 +3417,15 @@
         <v>8</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="85" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>7</v>
@@ -3174,15 +3434,15 @@
         <v>8</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="86" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>7</v>
@@ -3191,15 +3451,15 @@
         <v>8</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="87" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C87" s="3" t="s">
         <v>7</v>
@@ -3208,32 +3468,32 @@
         <v>8</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="88" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E88" s="2" t="s">
         <v>204</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="C88" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="89" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>7</v>
@@ -3242,32 +3502,32 @@
         <v>8</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="90" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E90" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="91" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C91" s="3" t="s">
         <v>7</v>
@@ -3276,32 +3536,32 @@
         <v>8</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="92" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E92" s="2" t="s">
         <v>214</v>
-      </c>
-      <c r="B92" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D92" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E92" s="2" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="93" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C93" s="3" t="s">
         <v>7</v>
@@ -3310,15 +3570,15 @@
         <v>8</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="94" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C94" s="3" t="s">
         <v>7</v>
@@ -3327,15 +3587,15 @@
         <v>8</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="95" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C95" s="3" t="s">
         <v>7</v>
@@ -3344,15 +3604,15 @@
         <v>8</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="96" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>7</v>
@@ -3361,32 +3621,32 @@
         <v>8</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="97" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E97" s="2" t="s">
         <v>224</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D97" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E97" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="98" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C98" s="3" t="s">
         <v>7</v>
@@ -3395,15 +3655,15 @@
         <v>8</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="99" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C99" s="3" t="s">
         <v>7</v>
@@ -3412,15 +3672,15 @@
         <v>8</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="100" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>7</v>
@@ -3429,15 +3689,15 @@
         <v>8</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="101" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>7</v>
@@ -3446,66 +3706,66 @@
         <v>8</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="B102" s="4" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="C102" s="5" t="s">
+      <c r="B102" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="D102" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E102" s="4" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="4" t="s">
+      <c r="C102" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="B103" s="4" t="s">
+      <c r="B103" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="C103" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="D103" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E103" s="4" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="4" t="s">
+      <c r="C103" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="B104" s="4" t="s">
+      <c r="B104" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="C104" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="D104" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E104" s="4" t="s">
-        <v>223</v>
+      <c r="C104" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="105" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C105" s="3" t="s">
         <v>7</v>
@@ -3514,15 +3774,15 @@
         <v>8</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="106" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C106" s="3" t="s">
         <v>7</v>
@@ -3531,15 +3791,15 @@
         <v>8</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="107" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C107" s="3" t="s">
         <v>7</v>
@@ -3548,15 +3808,15 @@
         <v>8</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="108" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C108" s="3" t="s">
         <v>7</v>
@@ -3565,15 +3825,15 @@
         <v>8</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="109" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C109" s="3" t="s">
         <v>7</v>
@@ -3582,15 +3842,15 @@
         <v>8</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="110" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C110" s="3" t="s">
         <v>7</v>
@@ -3599,15 +3859,15 @@
         <v>8</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="111" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C111" s="3" t="s">
         <v>7</v>
@@ -3616,15 +3876,15 @@
         <v>8</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="112" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>7</v>
@@ -3633,24 +3893,24 @@
         <v>8</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="113" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E113" s="2" t="s">
         <v>265</v>
-      </c>
-      <c r="B113" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="C113" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="114" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3667,24 +3927,24 @@
         <v>8</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="115" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E115" s="2" t="s">
         <v>270</v>
-      </c>
-      <c r="B115" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="C115" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="116" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3701,24 +3961,24 @@
         <v>8</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="117" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E117" s="2" t="s">
         <v>275</v>
-      </c>
-      <c r="B117" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="C117" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D117" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E117" s="2" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="118" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3735,24 +3995,24 @@
         <v>8</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="119" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E119" s="2" t="s">
         <v>280</v>
-      </c>
-      <c r="B119" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="C119" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="120" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3769,15 +4029,15 @@
         <v>8</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="121" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>7</v>
@@ -3786,15 +4046,15 @@
         <v>8</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="122" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>7</v>
@@ -3803,15 +4063,15 @@
         <v>8</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="123" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C123" s="3" t="s">
         <v>7</v>
@@ -3820,15 +4080,15 @@
         <v>8</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="124" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C124" s="3" t="s">
         <v>7</v>
@@ -3837,15 +4097,15 @@
         <v>8</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="125" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C125" s="3" t="s">
         <v>7</v>
@@ -3854,15 +4114,15 @@
         <v>8</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="126" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C126" s="3" t="s">
         <v>7</v>
@@ -3871,15 +4131,15 @@
         <v>8</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="127" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C127" s="3" t="s">
         <v>7</v>
@@ -3888,15 +4148,15 @@
         <v>8</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="128" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C128" s="3" t="s">
         <v>7</v>
@@ -3905,15 +4165,15 @@
         <v>8</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="129" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C129" s="3" t="s">
         <v>7</v>
@@ -3922,15 +4182,15 @@
         <v>8</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="130" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C130" s="3" t="s">
         <v>7</v>
@@ -3939,15 +4199,15 @@
         <v>8</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="131" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C131" s="3" t="s">
         <v>7</v>
@@ -3956,15 +4216,15 @@
         <v>8</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="132" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C132" s="3" t="s">
         <v>7</v>
@@ -3973,15 +4233,15 @@
         <v>8</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="133" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C133" s="3" t="s">
         <v>7</v>
@@ -3990,15 +4250,15 @@
         <v>8</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="134" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C134" s="3" t="s">
         <v>7</v>
@@ -4007,15 +4267,15 @@
         <v>8</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="135" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C135" s="3" t="s">
         <v>7</v>
@@ -4024,15 +4284,15 @@
         <v>8</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="136" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C136" s="3" t="s">
         <v>7</v>
@@ -4041,15 +4301,15 @@
         <v>8</v>
       </c>
       <c r="E136" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="137" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C137" s="3" t="s">
         <v>7</v>
@@ -4058,15 +4318,15 @@
         <v>8</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="138" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C138" s="3" t="s">
         <v>7</v>
@@ -4075,15 +4335,15 @@
         <v>8</v>
       </c>
       <c r="E138" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="139" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C139" s="3" t="s">
         <v>7</v>
@@ -4092,15 +4352,15 @@
         <v>8</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="140" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C140" s="3" t="s">
         <v>7</v>
@@ -4109,15 +4369,15 @@
         <v>8</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="141" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C141" s="3" t="s">
         <v>7</v>
@@ -4126,15 +4386,15 @@
         <v>8</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="142" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C142" s="3" t="s">
         <v>7</v>
@@ -4143,15 +4403,15 @@
         <v>8</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="143" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C143" s="3" t="s">
         <v>7</v>
@@ -4160,15 +4420,15 @@
         <v>8</v>
       </c>
       <c r="E143" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="144" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C144" s="3" t="s">
         <v>7</v>
@@ -4177,15 +4437,15 @@
         <v>8</v>
       </c>
       <c r="E144" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="145" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C145" s="3" t="s">
         <v>7</v>
@@ -4194,24 +4454,24 @@
         <v>8</v>
       </c>
       <c r="E145" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="146" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E146" s="2" t="s">
         <v>360</v>
-      </c>
-      <c r="B146" s="2" t="s">
-        <v>361</v>
-      </c>
-      <c r="C146" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D146" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E146" s="2" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="147" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4228,7 +4488,7 @@
         <v>8</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="148" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4245,24 +4505,24 @@
         <v>8</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
     </row>
     <row r="149" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E149" s="2" t="s">
         <v>367</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="C149" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D149" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E149" s="2" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="150" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4279,7 +4539,7 @@
         <v>8</v>
       </c>
       <c r="E150" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="151" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4296,24 +4556,24 @@
         <v>8</v>
       </c>
       <c r="E151" s="2" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
     </row>
     <row r="152" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E152" s="2" t="s">
         <v>374</v>
-      </c>
-      <c r="B152" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="C152" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D152" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E152" s="2" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="153" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4330,7 +4590,7 @@
         <v>8</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="154" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4347,15 +4607,15 @@
         <v>8</v>
       </c>
       <c r="E154" s="2" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
     </row>
     <row r="155" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C155" s="3" t="s">
         <v>7</v>
@@ -4364,15 +4624,15 @@
         <v>8</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="156" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C156" s="3" t="s">
         <v>7</v>
@@ -4381,15 +4641,15 @@
         <v>8</v>
       </c>
       <c r="E156" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="157" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C157" s="3" t="s">
         <v>7</v>
@@ -4398,15 +4658,15 @@
         <v>8</v>
       </c>
       <c r="E157" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="158" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C158" s="3" t="s">
         <v>7</v>
@@ -4415,15 +4675,15 @@
         <v>8</v>
       </c>
       <c r="E158" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="159" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C159" s="3" t="s">
         <v>7</v>
@@ -4432,15 +4692,15 @@
         <v>8</v>
       </c>
       <c r="E159" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="160" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C160" s="3" t="s">
         <v>7</v>
@@ -4449,15 +4709,15 @@
         <v>8</v>
       </c>
       <c r="E160" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="161" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C161" s="3" t="s">
         <v>7</v>
@@ -4466,15 +4726,15 @@
         <v>8</v>
       </c>
       <c r="E161" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="162" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C162" s="3" t="s">
         <v>7</v>
@@ -4483,15 +4743,15 @@
         <v>8</v>
       </c>
       <c r="E162" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="163" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C163" s="3" t="s">
         <v>7</v>
@@ -4500,66 +4760,66 @@
         <v>8</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="164" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="B164" s="2" t="s">
+    </row>
+    <row r="164" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="4" t="s">
         <v>409</v>
       </c>
-      <c r="C164" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D164" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E164" s="2" t="s">
+      <c r="B164" s="4" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="165" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A165" s="2" t="s">
+      <c r="C164" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="B165" s="2" t="s">
+      <c r="D164" s="4" t="s">
         <v>412</v>
       </c>
-      <c r="C165" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D165" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E165" s="2" t="s">
+      <c r="E164" s="4" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="166" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="2" t="s">
+    <row r="165" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="4" t="s">
         <v>414</v>
       </c>
-      <c r="B166" s="2" t="s">
+      <c r="B165" s="4" t="s">
         <v>415</v>
       </c>
-      <c r="C166" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D166" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E166" s="2" t="s">
+      <c r="C165" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="D165" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="E165" s="4" t="s">
         <v>416</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="C166" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="D166" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="E166" s="4" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="167" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="C167" s="3" t="s">
         <v>7</v>
@@ -4568,15 +4828,15 @@
         <v>8</v>
       </c>
       <c r="E167" s="2" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
     </row>
     <row r="168" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="C168" s="3" t="s">
         <v>7</v>
@@ -4585,15 +4845,15 @@
         <v>8</v>
       </c>
       <c r="E168" s="2" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="169" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C169" s="3" t="s">
         <v>7</v>
@@ -4602,15 +4862,15 @@
         <v>8</v>
       </c>
       <c r="E169" s="2" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="170" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="C170" s="3" t="s">
         <v>7</v>
@@ -4619,24 +4879,534 @@
         <v>8</v>
       </c>
       <c r="E170" s="2" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="172" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A172" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="B172" s="6" t="s">
-        <v>430</v>
-      </c>
-      <c r="C172" s="6" t="s">
         <v>431</v>
       </c>
-      <c r="D172" s="6" t="s">
+    </row>
+    <row r="171" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A171" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="E172" s="6" t="s">
+      <c r="B171" s="2" t="s">
         <v>433</v>
+      </c>
+      <c r="C171" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E171" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C172" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E172" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A173" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="C173" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E173" s="2" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A174" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C174" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A175" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="B175" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="C175" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E175" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C176" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E176" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="C177" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E177" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E178" s="2" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="B179" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="C179" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D179" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E179" s="2" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="B180" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D180" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E180" s="2" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="B181" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="C181" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D181" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E181" s="2" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="B182" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="C182" s="7" t="s">
+        <v>463</v>
+      </c>
+      <c r="D182" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E182" s="6" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B183" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="C183" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D183" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E183" s="2" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="B184" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="C184" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D184" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E184" s="2" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="B185" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="C185" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D185" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E185" s="2" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="B186" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="C186" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="D186" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="E186" s="4" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="B187" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="C187" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D187" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E187" s="2" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="B188" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="C188" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D188" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E188" s="2" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="B189" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="C189" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D189" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E189" s="2" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="B190" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="C190" s="7" t="s">
+        <v>463</v>
+      </c>
+      <c r="D190" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E190" s="6" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B191" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="C191" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D191" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E191" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="B192" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="C192" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D192" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E192" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="B193" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C193" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D193" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E193" s="2" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="C194" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D194" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E194" s="2" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="B195" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C195" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D195" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E195" s="2" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="B196" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C196" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D196" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E196" s="2" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="B197" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C197" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D197" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E197" s="2" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="C198" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D198" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E198" s="2" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="B199" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="C199" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D199" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E199" s="2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="B200" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="C200" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D200" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E200" s="2" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A202" s="8" t="s">
+        <v>513</v>
+      </c>
+      <c r="B202" s="8" t="s">
+        <v>514</v>
+      </c>
+      <c r="C202" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="D202" s="8" t="s">
+        <v>516</v>
+      </c>
+      <c r="E202" s="8" t="s">
+        <v>517</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: useParams from-id still referenced old /library/$id after rename
</commit_message>
<xml_diff>
--- a/tests/reports/selenium-report.xlsx
+++ b/tests/reports/selenium-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="536">
   <si>
     <t>Test ID</t>
   </si>
@@ -40,7 +40,7 @@
     <t/>
   </si>
   <si>
-    <t>13/7/2026, 10:24:30 am</t>
+    <t>13/7/2026, 3:17:15 pm</t>
   </si>
   <si>
     <t>TC002</t>
@@ -55,7 +55,7 @@
     <t>Login page shows ChemoSense branding</t>
   </si>
   <si>
-    <t>13/7/2026, 10:24:34 am</t>
+    <t>13/7/2026, 3:17:19 pm</t>
   </si>
   <si>
     <t>TC004</t>
@@ -73,7 +73,7 @@
     <t>Invalid login shows error message</t>
   </si>
   <si>
-    <t>13/7/2026, 10:24:37 am</t>
+    <t>13/7/2026, 3:17:23 pm</t>
   </si>
   <si>
     <t>TC006</t>
@@ -82,7 +82,7 @@
     <t>Demo login redirects to dashboard</t>
   </si>
   <si>
-    <t>13/7/2026, 10:24:48 am</t>
+    <t>13/7/2026, 3:17:33 pm</t>
   </si>
   <si>
     <t>TC007</t>
@@ -91,6 +91,9 @@
     <t>Dashboard visible after demo login</t>
   </si>
   <si>
+    <t>13/7/2026, 3:17:34 pm</t>
+  </si>
+  <si>
     <t>TC008</t>
   </si>
   <si>
@@ -118,7 +121,7 @@
     <t>Dashboard Total Scans card</t>
   </si>
   <si>
-    <t>13/7/2026, 10:24:52 am</t>
+    <t>13/7/2026, 3:17:37 pm</t>
   </si>
   <si>
     <t>TC012</t>
@@ -181,7 +184,7 @@
     <t>Scan page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:24:55 am</t>
+    <t>13/7/2026, 3:17:41 pm</t>
   </si>
   <si>
     <t>TC022</t>
@@ -208,16 +211,13 @@
     <t>Scan textarea accepts input</t>
   </si>
   <si>
-    <t>13/7/2026, 10:24:56 am</t>
-  </si>
-  <si>
     <t>TC026</t>
   </si>
   <si>
     <t>Symptom scan returns AI results</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:09 am</t>
+    <t>13/7/2026, 3:17:55 pm</t>
   </si>
   <si>
     <t>TC027</t>
@@ -256,7 +256,7 @@
     <t>Mode B biomarker mode works</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:14 am</t>
+    <t>13/7/2026, 3:18:00 pm</t>
   </si>
   <si>
     <t>TC033</t>
@@ -265,7 +265,7 @@
     <t>Cases list page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:18 am</t>
+    <t>13/7/2026, 3:18:04 pm</t>
   </si>
   <si>
     <t>TC034</t>
@@ -304,7 +304,7 @@
     <t>Case detail page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:22 am</t>
+    <t>13/7/2026, 3:18:08 pm</t>
   </si>
   <si>
     <t>TC040</t>
@@ -331,7 +331,7 @@
     <t>Patients page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:25 am</t>
+    <t>13/7/2026, 3:18:12 pm</t>
   </si>
   <si>
     <t>TC044</t>
@@ -352,7 +352,7 @@
     <t>Patient selection shows timeline</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:29 am</t>
+    <t>13/7/2026, 3:18:15 pm</t>
   </si>
   <si>
     <t>TC047</t>
@@ -373,7 +373,7 @@
     <t>Alerts page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:32 am</t>
+    <t>13/7/2026, 3:18:18 pm</t>
   </si>
   <si>
     <t>TC050</t>
@@ -400,7 +400,7 @@
     <t>Bell icon links to alerts</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:36 am</t>
+    <t>13/7/2026, 3:18:22 pm</t>
   </si>
   <si>
     <t>TC054</t>
@@ -409,7 +409,7 @@
     <t>Sensors page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:42 am</t>
+    <t>13/7/2026, 3:18:26 pm</t>
   </si>
   <si>
     <t>TC055</t>
@@ -466,7 +466,7 @@
     <t>Simulator page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:45 am</t>
+    <t>13/7/2026, 3:18:29 pm</t>
   </si>
   <si>
     <t>TC064</t>
@@ -475,9 +475,6 @@
     <t>DPV Colorimetric platform visible</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:46 am</t>
-  </si>
-  <si>
     <t>TC065</t>
   </si>
   <si>
@@ -514,7 +511,7 @@
     <t>Simulator run scan generates live signal</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:56 am</t>
+    <t>13/7/2026, 3:18:39 pm</t>
   </si>
   <si>
     <t>TC071</t>
@@ -523,7 +520,7 @@
     <t>Pathogen library loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:25:59 am</t>
+    <t>13/7/2026, 3:18:43 pm</t>
   </si>
   <si>
     <t>TC072</t>
@@ -556,7 +553,10 @@
     <t>Pathogen detail page loads on click</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:02 am</t>
+    <t>SKIP</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:18:46 pm</t>
   </si>
   <si>
     <t>TC077</t>
@@ -565,7 +565,7 @@
     <t>Compare page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:07 am</t>
+    <t>13/7/2026, 3:18:49 pm</t>
   </si>
   <si>
     <t>TC078</t>
@@ -592,7 +592,7 @@
     <t>Analytics page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:10 am</t>
+    <t>13/7/2026, 3:18:52 pm</t>
   </si>
   <si>
     <t>TC082</t>
@@ -601,6 +601,9 @@
     <t>Analytics infection timeline visible</t>
   </si>
   <si>
+    <t>13/7/2026, 3:18:53 pm</t>
+  </si>
+  <si>
     <t>TC083</t>
   </si>
   <si>
@@ -625,7 +628,7 @@
     <t>History page shows scan records</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:14 am</t>
+    <t>13/7/2026, 3:18:56 pm</t>
   </si>
   <si>
     <t>TC087</t>
@@ -640,7 +643,7 @@
     <t>Outbreaks page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:18 am</t>
+    <t>13/7/2026, 3:19:00 pm</t>
   </si>
   <si>
     <t>TC089</t>
@@ -655,7 +658,7 @@
     <t>Settings page loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:21 am</t>
+    <t>13/7/2026, 3:19:03 pm</t>
   </si>
   <si>
     <t>TC091</t>
@@ -685,7 +688,7 @@
     <t>TC101</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:25 am</t>
+    <t>13/7/2026, 3:19:07 pm</t>
   </si>
   <si>
     <t>TC102</t>
@@ -736,7 +739,10 @@
     <t>Pathogen detail card #1 renders</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:31 am</t>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:19:13 pm</t>
   </si>
   <si>
     <t>TC110</t>
@@ -745,7 +751,7 @@
     <t>Pathogen detail card #2 renders</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:33 am</t>
+    <t>13/7/2026, 3:19:15 pm</t>
   </si>
   <si>
     <t>TC111</t>
@@ -754,7 +760,7 @@
     <t>Pathogen detail card #3 renders</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:36 am</t>
+    <t>13/7/2026, 3:19:18 pm</t>
   </si>
   <si>
     <t>TC112</t>
@@ -763,7 +769,7 @@
     <t>Pathogen detail card #4 renders</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:39 am</t>
+    <t>13/7/2026, 3:19:20 pm</t>
   </si>
   <si>
     <t>TC113</t>
@@ -772,7 +778,7 @@
     <t>Pathogen detail card #5 renders</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:41 am</t>
+    <t>13/7/2026, 3:19:23 pm</t>
   </si>
   <si>
     <t>TC114</t>
@@ -781,7 +787,7 @@
     <t>Pathogen detail card #6 renders</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:44 am</t>
+    <t>13/7/2026, 3:19:25 pm</t>
   </si>
   <si>
     <t>TC115</t>
@@ -790,7 +796,7 @@
     <t>Pathogen detail card #7 renders</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:46 am</t>
+    <t>13/7/2026, 3:19:28 pm</t>
   </si>
   <si>
     <t>TC116</t>
@@ -799,7 +805,7 @@
     <t>Pathogen detail card #8 renders</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:49 am</t>
+    <t>13/7/2026, 3:19:31 pm</t>
   </si>
   <si>
     <t>TC117</t>
@@ -808,7 +814,7 @@
     <t>Compare Pseudomonas aeruginosa vs Staphylococcus aureus shows QS</t>
   </si>
   <si>
-    <t>13/7/2026, 10:26:55 am</t>
+    <t>13/7/2026, 3:19:37 pm</t>
   </si>
   <si>
     <t>TC118</t>
@@ -823,7 +829,7 @@
     <t>Compare Klebsiella pneumoniae vs Escherichia coli shows QS</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:04 am</t>
+    <t>13/7/2026, 3:19:42 pm</t>
   </si>
   <si>
     <t>TC120</t>
@@ -838,7 +844,7 @@
     <t>Compare Acinetobacter baumannii vs Enterococcus faecium shows QS</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:13 am</t>
+    <t>13/7/2026, 3:19:47 pm</t>
   </si>
   <si>
     <t>TC122</t>
@@ -853,7 +859,7 @@
     <t>Compare Mycobacterium tuberculosis vs Vibrio cholerae shows QS</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:19 am</t>
+    <t>13/7/2026, 3:19:52 pm</t>
   </si>
   <si>
     <t>TC124</t>
@@ -868,7 +874,7 @@
     <t>Simulator DPV platform selectable, shows LOD</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:24 am</t>
+    <t>13/7/2026, 3:19:57 pm</t>
   </si>
   <si>
     <t>TC126</t>
@@ -877,7 +883,7 @@
     <t>Simulator Piezoelectric platform selectable, shows LOD</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:25 am</t>
+    <t>13/7/2026, 3:19:58 pm</t>
   </si>
   <si>
     <t>TC127</t>
@@ -886,7 +892,7 @@
     <t>Simulator FRET platform selectable, shows LOD</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:26 am</t>
+    <t>13/7/2026, 3:19:59 pm</t>
   </si>
   <si>
     <t>TC128</t>
@@ -895,7 +901,7 @@
     <t>Simulator Lateral Flow platform selectable, shows LOD</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:27 am</t>
+    <t>13/7/2026, 3:20:00 pm</t>
   </si>
   <si>
     <t>TC129</t>
@@ -904,7 +910,7 @@
     <t>Simulator MIP platform selectable, shows LOD</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:28 am</t>
+    <t>13/7/2026, 3:20:01 pm</t>
   </si>
   <si>
     <t>TC130</t>
@@ -913,7 +919,7 @@
     <t>Route /dashboard loads (Dashboard)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:32 am</t>
+    <t>13/7/2026, 3:20:04 pm</t>
   </si>
   <si>
     <t>TC131</t>
@@ -922,7 +928,7 @@
     <t>Route /scan loads (Scan)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:38 am</t>
+    <t>13/7/2026, 3:20:08 pm</t>
   </si>
   <si>
     <t>TC132</t>
@@ -931,7 +937,7 @@
     <t>Route /cases loads (Case)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:42 am</t>
+    <t>13/7/2026, 3:20:12 pm</t>
   </si>
   <si>
     <t>TC133</t>
@@ -940,7 +946,7 @@
     <t>Route /patients loads (Patient)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:45 am</t>
+    <t>13/7/2026, 3:20:15 pm</t>
   </si>
   <si>
     <t>TC134</t>
@@ -949,7 +955,7 @@
     <t>Route /alerts loads (Alert)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:49 am</t>
+    <t>13/7/2026, 3:20:18 pm</t>
   </si>
   <si>
     <t>TC135</t>
@@ -958,7 +964,7 @@
     <t>Route /sensors loads (Sensor)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:56 am</t>
+    <t>13/7/2026, 3:20:22 pm</t>
   </si>
   <si>
     <t>TC136</t>
@@ -967,7 +973,7 @@
     <t>Route /simulator loads (Simulator)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:27:59 am</t>
+    <t>13/7/2026, 3:20:25 pm</t>
   </si>
   <si>
     <t>TC137</t>
@@ -976,7 +982,7 @@
     <t>Route /library loads (Pathogen)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:03 am</t>
+    <t>13/7/2026, 3:20:29 pm</t>
   </si>
   <si>
     <t>TC138</t>
@@ -985,7 +991,7 @@
     <t>Route /compare loads (Compare)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:06 am</t>
+    <t>13/7/2026, 3:20:33 pm</t>
   </si>
   <si>
     <t>TC139</t>
@@ -994,7 +1000,7 @@
     <t>Route /analytics loads (Analytics)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:10 am</t>
+    <t>13/7/2026, 3:20:36 pm</t>
   </si>
   <si>
     <t>TC140</t>
@@ -1003,7 +1009,7 @@
     <t>Route /history loads (History)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:13 am</t>
+    <t>13/7/2026, 3:20:40 pm</t>
   </si>
   <si>
     <t>TC141</t>
@@ -1012,7 +1018,7 @@
     <t>Route /outbreaks loads (Outbreak)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:17 am</t>
+    <t>13/7/2026, 3:20:44 pm</t>
   </si>
   <si>
     <t>TC142</t>
@@ -1021,7 +1027,7 @@
     <t>Route /settings loads (Settings)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:22 am</t>
+    <t>13/7/2026, 3:20:47 pm</t>
   </si>
   <si>
     <t>TC143</t>
@@ -1030,7 +1036,7 @@
     <t>Forgot-password valid id shows reset info</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:29 am</t>
+    <t>13/7/2026, 3:20:53 pm</t>
   </si>
   <si>
     <t>TC144</t>
@@ -1039,7 +1045,7 @@
     <t>Forgot-password invalid id shows error</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:35 am</t>
+    <t>13/7/2026, 3:20:58 pm</t>
   </si>
   <si>
     <t>TC145</t>
@@ -1048,7 +1054,7 @@
     <t>Cases search filters to empty for gibberish query</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:39 am</t>
+    <t>13/7/2026, 3:21:02 pm</t>
   </si>
   <si>
     <t>TC146</t>
@@ -1057,7 +1063,7 @@
     <t>Cases status filter controls present</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:43 am</t>
+    <t>13/7/2026, 3:21:06 pm</t>
   </si>
   <si>
     <t>TC147</t>
@@ -1066,7 +1072,7 @@
     <t>History has risk/patient filter dropdown</t>
   </si>
   <si>
-    <t>13/7/2026, 10:28:46 am</t>
+    <t>13/7/2026, 3:21:09 pm</t>
   </si>
   <si>
     <t>TC148</t>
@@ -1075,7 +1081,7 @@
     <t>Alerts has mark-read control(s)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:04 am</t>
+    <t>13/7/2026, 3:21:13 pm</t>
   </si>
   <si>
     <t>TC149</t>
@@ -1084,7 +1090,7 @@
     <t>Theme toggle changes html class</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:08 am</t>
+    <t>13/7/2026, 3:21:17 pm</t>
   </si>
   <si>
     <t>TC150</t>
@@ -1093,7 +1099,7 @@
     <t>Case #1 has PDF/Download</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:16 am</t>
+    <t>13/7/2026, 3:21:24 pm</t>
   </si>
   <si>
     <t>TC151</t>
@@ -1114,7 +1120,7 @@
     <t>Case #2 has PDF/Download</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:19 am</t>
+    <t>13/7/2026, 3:21:27 pm</t>
   </si>
   <si>
     <t>TC154</t>
@@ -1135,7 +1141,7 @@
     <t>Case #3 has PDF/Download</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:22 am</t>
+    <t>13/7/2026, 3:21:29 pm</t>
   </si>
   <si>
     <t>TC157</t>
@@ -1156,7 +1162,7 @@
     <t>Patient row #1 timeline loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:27 am</t>
+    <t>13/7/2026, 3:21:35 pm</t>
   </si>
   <si>
     <t>TC160</t>
@@ -1165,7 +1171,7 @@
     <t>Patient row #2 timeline loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:29 am</t>
+    <t>13/7/2026, 3:21:37 pm</t>
   </si>
   <si>
     <t>TC161</t>
@@ -1174,7 +1180,7 @@
     <t>Patient row #3 timeline loads</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:30 am</t>
+    <t>13/7/2026, 3:21:38 pm</t>
   </si>
   <si>
     <t>TC162</t>
@@ -1183,7 +1189,7 @@
     <t>Nonexistent case id handled gracefully</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:33 am</t>
+    <t>13/7/2026, 3:21:41 pm</t>
   </si>
   <si>
     <t>TC163</t>
@@ -1192,7 +1198,7 @@
     <t>Nonexistent patient id handled gracefully</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:36 am</t>
+    <t>13/7/2026, 3:21:44 pm</t>
   </si>
   <si>
     <t>TC164</t>
@@ -1201,7 +1207,7 @@
     <t>Unauthenticated access to /dashboard redirects to login</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:39 am</t>
+    <t>13/7/2026, 3:21:47 pm</t>
   </si>
   <si>
     <t>TC165</t>
@@ -1210,7 +1216,7 @@
     <t>Unauthenticated access to /cases redirects to login</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:42 am</t>
+    <t>13/7/2026, 3:21:51 pm</t>
   </si>
   <si>
     <t>TC166</t>
@@ -1219,7 +1225,7 @@
     <t>Unauthenticated access to /patients redirects to login</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:46 am</t>
+    <t>13/7/2026, 3:21:54 pm</t>
   </si>
   <si>
     <t>TC167</t>
@@ -1228,7 +1234,7 @@
     <t>Unauthenticated access to /alerts redirects to login</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:49 am</t>
+    <t>13/7/2026, 3:21:58 pm</t>
   </si>
   <si>
     <t>TC168</t>
@@ -1237,7 +1243,7 @@
     <t>Unauthenticated access to /settings redirects to login</t>
   </si>
   <si>
-    <t>13/7/2026, 10:29:52 am</t>
+    <t>13/7/2026, 3:22:01 pm</t>
   </si>
   <si>
     <t>TC169</t>
@@ -1246,13 +1252,10 @@
     <t>Register as technician reaches dashboard</t>
   </si>
   <si>
-    <t>FAIL</t>
-  </si>
-  <si>
     <t>https://chemosense-app.onrender.com/login?demo=false</t>
   </si>
   <si>
-    <t>13/7/2026, 10:30:09 am</t>
+    <t>13/7/2026, 3:22:19 pm</t>
   </si>
   <si>
     <t>TC170</t>
@@ -1261,172 +1264,160 @@
     <t>Register as doctor reaches dashboard</t>
   </si>
   <si>
-    <t>13/7/2026, 10:30:17 am</t>
+    <t>13/7/2026, 3:22:29 pm</t>
   </si>
   <si>
     <t>TC171</t>
   </si>
   <si>
-    <t>Register as admin reaches dashboard</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:25 am</t>
+    <t>Change-password rejects wrong current password</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:43 pm</t>
   </si>
   <si>
     <t>TC172</t>
   </si>
   <si>
-    <t>Change-password rejects wrong current password</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:39 am</t>
+    <t>Mode B biomarker search available (context: Pseudomonas aeruginosa)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:48 pm</t>
   </si>
   <si>
     <t>TC173</t>
   </si>
   <si>
-    <t>Mode B biomarker search available (context: Pseudomonas aeruginosa)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:44 am</t>
+    <t>Mode B biomarker search available (context: Staphylococcus aureus)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:49 pm</t>
   </si>
   <si>
     <t>TC174</t>
   </si>
   <si>
-    <t>Mode B biomarker search available (context: Staphylococcus aureus)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:45 am</t>
+    <t>Mode B biomarker search available (context: Escherichia coli)</t>
   </si>
   <si>
     <t>TC175</t>
   </si>
   <si>
-    <t>Mode B biomarker search available (context: Escherichia coli)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:46 am</t>
+    <t>Mode B biomarker search available (context: Klebsiella pneumoniae)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:50 pm</t>
   </si>
   <si>
     <t>TC176</t>
   </si>
   <si>
-    <t>Mode B biomarker search available (context: Klebsiella pneumoniae)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:47 am</t>
+    <t>Mode B biomarker search available (context: Acinetobacter baumannii)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:51 pm</t>
   </si>
   <si>
     <t>TC177</t>
   </si>
   <si>
-    <t>Mode B biomarker search available (context: Acinetobacter baumannii)</t>
+    <t>Mode B biomarker search available (context: Enterococcus faecium)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:52 pm</t>
   </si>
   <si>
     <t>TC178</t>
   </si>
   <si>
-    <t>Mode B biomarker search available (context: Enterococcus faecium)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:48 am</t>
+    <t>Mode B biomarker search available (context: Mycobacterium tuberculosis)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:53 pm</t>
   </si>
   <si>
     <t>TC179</t>
   </si>
   <si>
-    <t>Mode B biomarker search available (context: Mycobacterium tuberculosis)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:49 am</t>
+    <t>Mode B biomarker search available (context: Vibrio cholerae)</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:54 pm</t>
   </si>
   <si>
     <t>TC180</t>
   </si>
   <si>
-    <t>Mode B biomarker search available (context: Vibrio cholerae)</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:50 am</t>
+    <t>Analytics quick-fill button #1 clickable</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:58 pm</t>
   </si>
   <si>
     <t>TC181</t>
   </si>
   <si>
-    <t>Analytics quick-fill button #1 clickable</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:54 am</t>
+    <t>Analytics quick-fill button #2 clickable</t>
   </si>
   <si>
     <t>TC182</t>
   </si>
   <si>
-    <t>Analytics quick-fill button #2 clickable</t>
+    <t>Analytics quick-fill button #3 clickable</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:22:59 pm</t>
   </si>
   <si>
     <t>TC183</t>
   </si>
   <si>
-    <t>Analytics quick-fill button #3 clickable</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:55 am</t>
+    <t>Analytics quick-fill button #4 clickable</t>
   </si>
   <si>
     <t>TC184</t>
   </si>
   <si>
-    <t>Analytics quick-fill button #4 clickable</t>
+    <t>Outbreaks may reference Pseudomonas aeruginosa</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:23:14 pm</t>
   </si>
   <si>
     <t>TC185</t>
   </si>
   <si>
-    <t>Outbreaks may reference Pseudomonas aeruginosa</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:30:59 am</t>
+    <t>Outbreaks may reference Staphylococcus aureus</t>
   </si>
   <si>
     <t>TC186</t>
   </si>
   <si>
-    <t>Outbreaks may reference Staphylococcus aureus</t>
+    <t>Outbreaks page loaded (no Escherichia coli mention, acceptable)</t>
   </si>
   <si>
     <t>TC187</t>
   </si>
   <si>
-    <t>Outbreaks page loaded (no Escherichia coli mention, acceptable)</t>
-  </si>
-  <si>
-    <t>SKIP</t>
+    <t>Outbreaks may reference Klebsiella pneumoniae</t>
   </si>
   <si>
     <t>TC188</t>
   </si>
   <si>
-    <t>Outbreaks may reference Klebsiella pneumoniae</t>
+    <t>Outbreaks may reference Acinetobacter baumannii</t>
   </si>
   <si>
     <t>TC189</t>
   </si>
   <si>
-    <t>Outbreaks may reference Acinetobacter baumannii</t>
-  </si>
-  <si>
-    <t>TC190</t>
-  </si>
-  <si>
     <t>Ward heatmap renders grid cells</t>
   </si>
   <si>
-    <t>13/7/2026, 10:31:02 am</t>
-  </si>
-  <si>
-    <t>TC192</t>
+    <t>13/7/2026, 3:23:17 pm</t>
+  </si>
+  <si>
+    <t>TC191</t>
   </si>
   <si>
     <t>Sensor add form</t>
@@ -1436,67 +1427,130 @@
   (Session info: chrome=150.0.7871.49)</t>
   </si>
   <si>
-    <t>13/7/2026, 10:31:08 am</t>
+    <t>13/7/2026, 3:23:23 pm</t>
+  </si>
+  <si>
+    <t>TC192</t>
+  </si>
+  <si>
+    <t>Dashboard shows Critical risk tier</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:23:27 pm</t>
   </si>
   <si>
     <t>TC193</t>
   </si>
   <si>
-    <t>Dashboard shows Critical risk tier</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:31:11 am</t>
+    <t>Dashboard shows High risk tier</t>
   </si>
   <si>
     <t>TC194</t>
   </si>
   <si>
-    <t>Dashboard shows High risk tier</t>
+    <t>Dashboard shows Moderate risk tier</t>
   </si>
   <si>
     <t>TC195</t>
   </si>
   <si>
-    <t>Dashboard shows Moderate risk tier</t>
+    <t>Dashboard shows Low risk tier</t>
   </si>
   <si>
     <t>TC196</t>
   </si>
   <si>
-    <t>Dashboard shows Low risk tier</t>
+    <t>Cases list shows Open status pill</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:23:30 pm</t>
   </si>
   <si>
     <t>TC197</t>
   </si>
   <si>
-    <t>Cases list shows Open status pill</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:31:15 am</t>
+    <t>Cases list shows Closed status pill</t>
   </si>
   <si>
     <t>TC198</t>
   </si>
   <si>
-    <t>Cases list shows Closed status pill</t>
+    <t>Settings profile field is editable</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:23:34 pm</t>
   </si>
   <si>
     <t>TC199</t>
   </si>
   <si>
-    <t>Settings profile field is editable</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:31:18 am</t>
+    <t>Sign out then demo sign-in round trip works</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:23:49 pm</t>
   </si>
   <si>
     <t>TC200</t>
   </si>
   <si>
-    <t>Sign out then demo sign-in round trip works</t>
-  </si>
-  <si>
-    <t>13/7/2026, 10:31:33 am</t>
+    <t>Route / (landing) renders non-empty content</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:23:52 pm</t>
+  </si>
+  <si>
+    <t>TC201</t>
+  </si>
+  <si>
+    <t>Route /login (login) renders non-empty content</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:23:56 pm</t>
+  </si>
+  <si>
+    <t>TC202</t>
+  </si>
+  <si>
+    <t>Scan Mode A tab clickable</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:24:00 pm</t>
+  </si>
+  <si>
+    <t>TC203</t>
+  </si>
+  <si>
+    <t>Scan Mode B tab clickable</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:24:01 pm</t>
+  </si>
+  <si>
+    <t>TC204</t>
+  </si>
+  <si>
+    <t>/dashboard loads consistently on repeat visit</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:24:07 pm</t>
+  </si>
+  <si>
+    <t>TC205</t>
+  </si>
+  <si>
+    <t>/cases loads consistently on repeat visit</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:24:15 pm</t>
+  </si>
+  <si>
+    <t>TC206</t>
+  </si>
+  <si>
+    <t>/patients loads consistently on repeat visit</t>
+  </si>
+  <si>
+    <t>13/7/2026, 3:24:22 pm</t>
   </si>
   <si>
     <t>TC095</t>
@@ -1505,7 +1559,7 @@
     <t>Backend health API healthy</t>
   </si>
   <si>
-    <t>13/7/2026, 10:31:35 am</t>
+    <t>13/7/2026, 3:24:24 pm</t>
   </si>
   <si>
     <t>TC096</t>
@@ -1514,7 +1568,7 @@
     <t>Backend dashboard API returns stats</t>
   </si>
   <si>
-    <t>13/7/2026, 10:31:40 am</t>
+    <t>13/7/2026, 3:24:28 pm</t>
   </si>
   <si>
     <t>TC097</t>
@@ -1523,7 +1577,7 @@
     <t>Backend scans API returns records</t>
   </si>
   <si>
-    <t>13/7/2026, 10:31:44 am</t>
+    <t>13/7/2026, 3:24:33 pm</t>
   </si>
   <si>
     <t>TC098</t>
@@ -1532,7 +1586,7 @@
     <t>Backend patients API returns data</t>
   </si>
   <si>
-    <t>13/7/2026, 10:31:48 am</t>
+    <t>13/7/2026, 3:24:37 pm</t>
   </si>
   <si>
     <t>TC099</t>
@@ -1541,7 +1595,7 @@
     <t>Backend outbreaks API returns data</t>
   </si>
   <si>
-    <t>13/7/2026, 10:31:51 am</t>
+    <t>13/7/2026, 3:24:40 pm</t>
   </si>
   <si>
     <t>TC100</t>
@@ -1550,22 +1604,22 @@
     <t>Sign out redirects to login</t>
   </si>
   <si>
-    <t>13/7/2026, 10:31:58 am</t>
+    <t>13/7/2026, 3:24:47 pm</t>
   </si>
   <si>
     <t>SUMMARY</t>
   </si>
   <si>
-    <t>Total:199</t>
-  </si>
-  <si>
-    <t>Pass:193</t>
-  </si>
-  <si>
-    <t>Fail:4</t>
-  </si>
-  <si>
-    <t>Skip:2</t>
+    <t>Total:205</t>
+  </si>
+  <si>
+    <t>Pass:191</t>
+  </si>
+  <si>
+    <t>Fail:11</t>
+  </si>
+  <si>
+    <t>Skip:3</t>
   </si>
 </sst>
 </file>
@@ -1607,12 +1661,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEE2E2"/>
+        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
+        <fgColor rgb="FFFEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -1982,7 +2036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E202"/>
+  <dimension ref="A1:E208"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2125,49 +2179,49 @@
         <v>8</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>7</v>
@@ -2176,15 +2230,15 @@
         <v>8</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>7</v>
@@ -2193,32 +2247,32 @@
         <v>8</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>7</v>
@@ -2227,15 +2281,15 @@
         <v>8</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>7</v>
@@ -2244,15 +2298,15 @@
         <v>8</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>7</v>
@@ -2261,15 +2315,15 @@
         <v>8</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>7</v>
@@ -2278,15 +2332,15 @@
         <v>8</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>7</v>
@@ -2295,15 +2349,15 @@
         <v>8</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>7</v>
@@ -2312,15 +2366,15 @@
         <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>7</v>
@@ -2329,15 +2383,15 @@
         <v>8</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>7</v>
@@ -2346,15 +2400,15 @@
         <v>8</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>7</v>
@@ -2363,32 +2417,32 @@
         <v>8</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>7</v>
@@ -2397,15 +2451,15 @@
         <v>8</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>7</v>
@@ -2414,15 +2468,15 @@
         <v>8</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>7</v>
@@ -2431,7 +2485,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3094,16 +3148,16 @@
         <v>8</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B66" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="C66" s="3" t="s">
         <v>7</v>
       </c>
@@ -3111,16 +3165,16 @@
         <v>8</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B67" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B67" s="2" t="s">
-        <v>158</v>
-      </c>
       <c r="C67" s="3" t="s">
         <v>7</v>
       </c>
@@ -3128,16 +3182,16 @@
         <v>8</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B68" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B68" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="C68" s="3" t="s">
         <v>7</v>
       </c>
@@ -3145,16 +3199,16 @@
         <v>8</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B69" s="2" t="s">
-        <v>162</v>
-      </c>
       <c r="C69" s="3" t="s">
         <v>7</v>
       </c>
@@ -3162,16 +3216,16 @@
         <v>8</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B70" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B70" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="C70" s="3" t="s">
         <v>7</v>
       </c>
@@ -3179,50 +3233,50 @@
         <v>8</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B71" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="C71" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B72" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="C72" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E72" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B73" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B73" s="2" t="s">
-        <v>172</v>
-      </c>
       <c r="C73" s="3" t="s">
         <v>7</v>
       </c>
@@ -3230,16 +3284,16 @@
         <v>8</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B74" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="C74" s="3" t="s">
         <v>7</v>
       </c>
@@ -3247,16 +3301,16 @@
         <v>8</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B75" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B75" s="2" t="s">
-        <v>176</v>
-      </c>
       <c r="C75" s="3" t="s">
         <v>7</v>
       </c>
@@ -3264,40 +3318,40 @@
         <v>8</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B76" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="C76" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C76" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="2" t="s">
+      <c r="B77" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="C77" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="C77" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E77" s="2" t="s">
+      <c r="D77" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E77" s="4" t="s">
         <v>181</v>
       </c>
     </row>
@@ -3400,32 +3454,32 @@
         <v>8</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="84" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E84" s="2" t="s">
         <v>196</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C84" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E84" s="2" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="85" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>7</v>
@@ -3434,15 +3488,15 @@
         <v>8</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="86" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>7</v>
@@ -3451,15 +3505,15 @@
         <v>8</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="87" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C87" s="3" t="s">
         <v>7</v>
@@ -3468,32 +3522,32 @@
         <v>8</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="88" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E88" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="C88" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="89" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>7</v>
@@ -3502,32 +3556,32 @@
         <v>8</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="90" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E90" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="91" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C91" s="3" t="s">
         <v>7</v>
@@ -3536,32 +3590,32 @@
         <v>8</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="92" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E92" s="2" t="s">
         <v>215</v>
-      </c>
-      <c r="B92" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D92" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E92" s="2" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="93" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C93" s="3" t="s">
         <v>7</v>
@@ -3570,15 +3624,15 @@
         <v>8</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="94" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C94" s="3" t="s">
         <v>7</v>
@@ -3587,15 +3641,15 @@
         <v>8</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="95" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C95" s="3" t="s">
         <v>7</v>
@@ -3604,15 +3658,15 @@
         <v>8</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="96" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>7</v>
@@ -3621,32 +3675,32 @@
         <v>8</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="97" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E97" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D97" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E97" s="2" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="98" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C98" s="3" t="s">
         <v>7</v>
@@ -3655,15 +3709,15 @@
         <v>8</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="99" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C99" s="3" t="s">
         <v>7</v>
@@ -3672,15 +3726,15 @@
         <v>8</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="100" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>7</v>
@@ -3689,15 +3743,15 @@
         <v>8</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="101" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>7</v>
@@ -3706,15 +3760,15 @@
         <v>8</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="102" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C102" s="3" t="s">
         <v>7</v>
@@ -3723,15 +3777,15 @@
         <v>8</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="103" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C103" s="3" t="s">
         <v>7</v>
@@ -3740,151 +3794,151 @@
         <v>8</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="B104" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="C104" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E104" s="2" t="s">
+      <c r="B104" s="6" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="2" t="s">
+      <c r="C104" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="B105" s="2" t="s">
+      <c r="D104" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E104" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="C105" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D105" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E105" s="2" t="s">
+    </row>
+    <row r="105" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="6" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="2" t="s">
+      <c r="B105" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="B106" s="2" t="s">
+      <c r="C105" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D105" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E105" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="C106" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E106" s="2" t="s">
+    </row>
+    <row r="106" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="6" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="2" t="s">
+      <c r="B106" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="B107" s="2" t="s">
+      <c r="C106" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D106" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E106" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="C107" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E107" s="2" t="s">
+    </row>
+    <row r="107" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="6" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="2" t="s">
+      <c r="B107" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="B108" s="2" t="s">
+      <c r="C107" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D107" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E107" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="C108" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D108" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E108" s="2" t="s">
+    </row>
+    <row r="108" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="6" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="2" t="s">
+      <c r="B108" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="B109" s="2" t="s">
+      <c r="C108" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D108" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E108" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="C109" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E109" s="2" t="s">
+    </row>
+    <row r="109" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="6" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="2" t="s">
+      <c r="B109" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="B110" s="2" t="s">
+      <c r="C109" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D109" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E109" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="C110" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E110" s="2" t="s">
+    </row>
+    <row r="110" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="6" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="2" t="s">
+      <c r="B110" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="B111" s="2" t="s">
+      <c r="C110" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D110" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E110" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="C111" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D111" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E111" s="2" t="s">
+    </row>
+    <row r="111" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="6" t="s">
         <v>262</v>
+      </c>
+      <c r="B111" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="C111" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D111" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E111" s="6" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="112" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>7</v>
@@ -3893,32 +3947,32 @@
         <v>8</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="113" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B113" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E113" s="2" t="s">
         <v>267</v>
-      </c>
-      <c r="C113" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="114" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C114" s="3" t="s">
         <v>7</v>
@@ -3927,32 +3981,32 @@
         <v>8</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="115" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B115" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E115" s="2" t="s">
         <v>272</v>
-      </c>
-      <c r="C115" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="116" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>7</v>
@@ -3961,32 +4015,32 @@
         <v>8</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="117" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B117" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E117" s="2" t="s">
         <v>277</v>
-      </c>
-      <c r="C117" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D117" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E117" s="2" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="118" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C118" s="3" t="s">
         <v>7</v>
@@ -3995,32 +4049,32 @@
         <v>8</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="119" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B119" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E119" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="C119" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="120" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C120" s="3" t="s">
         <v>7</v>
@@ -4029,15 +4083,15 @@
         <v>8</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="121" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>7</v>
@@ -4046,15 +4100,15 @@
         <v>8</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="122" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>7</v>
@@ -4063,15 +4117,15 @@
         <v>8</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="123" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C123" s="3" t="s">
         <v>7</v>
@@ -4080,15 +4134,15 @@
         <v>8</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="124" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C124" s="3" t="s">
         <v>7</v>
@@ -4097,15 +4151,15 @@
         <v>8</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="125" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C125" s="3" t="s">
         <v>7</v>
@@ -4114,15 +4168,15 @@
         <v>8</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="126" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C126" s="3" t="s">
         <v>7</v>
@@ -4131,15 +4185,15 @@
         <v>8</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="127" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C127" s="3" t="s">
         <v>7</v>
@@ -4148,15 +4202,15 @@
         <v>8</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="128" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C128" s="3" t="s">
         <v>7</v>
@@ -4165,15 +4219,15 @@
         <v>8</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="129" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C129" s="3" t="s">
         <v>7</v>
@@ -4182,15 +4236,15 @@
         <v>8</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="130" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C130" s="3" t="s">
         <v>7</v>
@@ -4199,15 +4253,15 @@
         <v>8</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="131" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C131" s="3" t="s">
         <v>7</v>
@@ -4216,15 +4270,15 @@
         <v>8</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="132" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C132" s="3" t="s">
         <v>7</v>
@@ -4233,15 +4287,15 @@
         <v>8</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="133" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C133" s="3" t="s">
         <v>7</v>
@@ -4250,15 +4304,15 @@
         <v>8</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="134" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C134" s="3" t="s">
         <v>7</v>
@@ -4267,15 +4321,15 @@
         <v>8</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="135" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C135" s="3" t="s">
         <v>7</v>
@@ -4284,15 +4338,15 @@
         <v>8</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="136" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C136" s="3" t="s">
         <v>7</v>
@@ -4301,15 +4355,15 @@
         <v>8</v>
       </c>
       <c r="E136" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="137" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C137" s="3" t="s">
         <v>7</v>
@@ -4318,15 +4372,15 @@
         <v>8</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="138" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C138" s="3" t="s">
         <v>7</v>
@@ -4335,15 +4389,15 @@
         <v>8</v>
       </c>
       <c r="E138" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="139" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C139" s="3" t="s">
         <v>7</v>
@@ -4352,15 +4406,15 @@
         <v>8</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="140" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C140" s="3" t="s">
         <v>7</v>
@@ -4369,15 +4423,15 @@
         <v>8</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="141" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C141" s="3" t="s">
         <v>7</v>
@@ -4386,15 +4440,15 @@
         <v>8</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="142" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C142" s="3" t="s">
         <v>7</v>
@@ -4403,15 +4457,15 @@
         <v>8</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="143" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C143" s="3" t="s">
         <v>7</v>
@@ -4420,15 +4474,15 @@
         <v>8</v>
       </c>
       <c r="E143" s="2" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="144" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C144" s="3" t="s">
         <v>7</v>
@@ -4437,15 +4491,15 @@
         <v>8</v>
       </c>
       <c r="E144" s="2" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="145" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C145" s="3" t="s">
         <v>7</v>
@@ -4454,32 +4508,32 @@
         <v>8</v>
       </c>
       <c r="E145" s="2" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="146" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B146" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E146" s="2" t="s">
         <v>362</v>
-      </c>
-      <c r="C146" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D146" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E146" s="2" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="147" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C147" s="3" t="s">
         <v>7</v>
@@ -4488,15 +4542,15 @@
         <v>8</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="148" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C148" s="3" t="s">
         <v>7</v>
@@ -4505,32 +4559,32 @@
         <v>8</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="149" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B149" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E149" s="2" t="s">
         <v>369</v>
-      </c>
-      <c r="C149" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D149" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E149" s="2" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="150" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C150" s="3" t="s">
         <v>7</v>
@@ -4539,15 +4593,15 @@
         <v>8</v>
       </c>
       <c r="E150" s="2" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="151" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C151" s="3" t="s">
         <v>7</v>
@@ -4556,32 +4610,32 @@
         <v>8</v>
       </c>
       <c r="E151" s="2" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="152" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B152" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E152" s="2" t="s">
         <v>376</v>
-      </c>
-      <c r="C152" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D152" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E152" s="2" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="153" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="C153" s="3" t="s">
         <v>7</v>
@@ -4590,15 +4644,15 @@
         <v>8</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="154" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C154" s="3" t="s">
         <v>7</v>
@@ -4607,15 +4661,15 @@
         <v>8</v>
       </c>
       <c r="E154" s="2" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="155" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C155" s="3" t="s">
         <v>7</v>
@@ -4624,15 +4678,15 @@
         <v>8</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="156" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="C156" s="3" t="s">
         <v>7</v>
@@ -4641,15 +4695,15 @@
         <v>8</v>
       </c>
       <c r="E156" s="2" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="157" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C157" s="3" t="s">
         <v>7</v>
@@ -4658,15 +4712,15 @@
         <v>8</v>
       </c>
       <c r="E157" s="2" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="158" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="C158" s="3" t="s">
         <v>7</v>
@@ -4675,15 +4729,15 @@
         <v>8</v>
       </c>
       <c r="E158" s="2" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="159" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C159" s="3" t="s">
         <v>7</v>
@@ -4692,15 +4746,15 @@
         <v>8</v>
       </c>
       <c r="E159" s="2" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="160" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C160" s="3" t="s">
         <v>7</v>
@@ -4709,15 +4763,15 @@
         <v>8</v>
       </c>
       <c r="E160" s="2" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="161" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="C161" s="3" t="s">
         <v>7</v>
@@ -4726,15 +4780,15 @@
         <v>8</v>
       </c>
       <c r="E161" s="2" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="162" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="C162" s="3" t="s">
         <v>7</v>
@@ -4743,15 +4797,15 @@
         <v>8</v>
       </c>
       <c r="E162" s="2" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="163" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C163" s="3" t="s">
         <v>7</v>
@@ -4760,66 +4814,66 @@
         <v>8</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="164" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="4" t="s">
-        <v>409</v>
-      </c>
-      <c r="B164" s="4" t="s">
         <v>410</v>
       </c>
-      <c r="C164" s="5" t="s">
+    </row>
+    <row r="164" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="6" t="s">
         <v>411</v>
       </c>
-      <c r="D164" s="4" t="s">
+      <c r="B164" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="E164" s="4" t="s">
+      <c r="C164" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D164" s="6" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="165" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A165" s="4" t="s">
+      <c r="E164" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="B165" s="4" t="s">
+    </row>
+    <row r="165" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="C165" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="D165" s="4" t="s">
-        <v>412</v>
-      </c>
-      <c r="E165" s="4" t="s">
+      <c r="B165" s="6" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="166" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="4" t="s">
+      <c r="C165" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D165" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="E165" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="B166" s="4" t="s">
+    </row>
+    <row r="166" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="C166" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="D166" s="4" t="s">
-        <v>412</v>
-      </c>
-      <c r="E166" s="4" t="s">
+      <c r="B166" s="2" t="s">
         <v>419</v>
+      </c>
+      <c r="C166" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>420</v>
       </c>
     </row>
     <row r="167" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C167" s="3" t="s">
         <v>7</v>
@@ -4828,15 +4882,15 @@
         <v>8</v>
       </c>
       <c r="E167" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="168" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C168" s="3" t="s">
         <v>7</v>
@@ -4845,24 +4899,24 @@
         <v>8</v>
       </c>
       <c r="E168" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="169" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="C169" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E169" s="2" t="s">
         <v>426</v>
-      </c>
-      <c r="B169" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="C169" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D169" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E169" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="170" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4913,15 +4967,15 @@
         <v>8</v>
       </c>
       <c r="E172" s="2" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
     </row>
     <row r="173" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C173" s="3" t="s">
         <v>7</v>
@@ -4930,15 +4984,15 @@
         <v>8</v>
       </c>
       <c r="E173" s="2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="174" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C174" s="3" t="s">
         <v>7</v>
@@ -4947,15 +5001,15 @@
         <v>8</v>
       </c>
       <c r="E174" s="2" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="175" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C175" s="3" t="s">
         <v>7</v>
@@ -4964,24 +5018,24 @@
         <v>8</v>
       </c>
       <c r="E175" s="2" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="176" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="C176" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E176" s="2" t="s">
         <v>446</v>
-      </c>
-      <c r="B176" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="C176" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D176" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E176" s="2" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="177" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4998,24 +5052,24 @@
         <v>8</v>
       </c>
       <c r="E177" s="2" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
     </row>
     <row r="178" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E178" s="2" t="s">
         <v>451</v>
-      </c>
-      <c r="B178" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="C178" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D178" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E178" s="2" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="179" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5032,67 +5086,67 @@
         <v>8</v>
       </c>
       <c r="E179" s="2" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
     </row>
     <row r="180" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="B180" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D180" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E180" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="B180" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="C180" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D180" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E180" s="2" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="181" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A181" s="2" t="s">
+    </row>
+    <row r="181" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="4" t="s">
         <v>459</v>
       </c>
-      <c r="B181" s="2" t="s">
+      <c r="B181" s="4" t="s">
         <v>460</v>
       </c>
-      <c r="C181" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D181" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E181" s="2" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="182" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A182" s="6" t="s">
+      <c r="C181" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D181" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E181" s="4" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="B182" s="6" t="s">
+      <c r="B182" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="C182" s="7" t="s">
-        <v>463</v>
-      </c>
-      <c r="D182" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E182" s="6" t="s">
-        <v>458</v>
+      <c r="C182" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D182" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E182" s="2" t="s">
+        <v>456</v>
       </c>
     </row>
     <row r="183" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="B183" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="B183" s="2" t="s">
-        <v>465</v>
-      </c>
       <c r="C183" s="3" t="s">
         <v>7</v>
       </c>
@@ -5100,57 +5154,57 @@
         <v>8</v>
       </c>
       <c r="E183" s="2" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="184" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="B184" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="B184" s="2" t="s">
+      <c r="C184" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D184" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E184" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="C184" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D184" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E184" s="2" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="185" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A185" s="2" t="s">
+    </row>
+    <row r="185" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="6" t="s">
         <v>468</v>
       </c>
-      <c r="B185" s="2" t="s">
+      <c r="B185" s="6" t="s">
         <v>469</v>
       </c>
-      <c r="C185" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D185" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E185" s="2" t="s">
+      <c r="C185" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D185" s="6" t="s">
         <v>470</v>
       </c>
-    </row>
-    <row r="186" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A186" s="4" t="s">
+      <c r="E185" s="6" t="s">
         <v>471</v>
       </c>
-      <c r="B186" s="4" t="s">
+    </row>
+    <row r="186" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="C186" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="D186" s="4" t="s">
+      <c r="B186" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="E186" s="4" t="s">
+      <c r="C186" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D186" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E186" s="2" t="s">
         <v>474</v>
       </c>
     </row>
@@ -5168,58 +5222,58 @@
         <v>8</v>
       </c>
       <c r="E187" s="2" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
     </row>
     <row r="188" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="B188" s="2" t="s">
         <v>478</v>
       </c>
-      <c r="B188" s="2" t="s">
+      <c r="C188" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D188" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E188" s="2" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="4" t="s">
         <v>479</v>
       </c>
-      <c r="C188" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D188" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E188" s="2" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A189" s="2" t="s">
+      <c r="B189" s="4" t="s">
         <v>480</v>
       </c>
-      <c r="B189" s="2" t="s">
+      <c r="C189" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D189" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E189" s="4" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="C189" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D189" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E189" s="2" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="190" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="6" t="s">
+      <c r="B190" s="2" t="s">
         <v>482</v>
       </c>
-      <c r="B190" s="6" t="s">
+      <c r="C190" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D190" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E190" s="2" t="s">
         <v>483</v>
-      </c>
-      <c r="C190" s="7" t="s">
-        <v>463</v>
-      </c>
-      <c r="D190" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E190" s="6" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="191" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5236,24 +5290,24 @@
         <v>8</v>
       </c>
       <c r="E191" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
     </row>
     <row r="192" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="B192" s="2" t="s">
         <v>487</v>
       </c>
-      <c r="B192" s="2" t="s">
+      <c r="C192" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D192" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E192" s="2" t="s">
         <v>488</v>
-      </c>
-      <c r="C192" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D192" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E192" s="2" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="193" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5392,21 +5446,123 @@
         <v>512</v>
       </c>
     </row>
-    <row r="202" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A202" s="8" t="s">
+    <row r="201" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="B202" s="8" t="s">
+      <c r="B201" s="2" t="s">
         <v>514</v>
       </c>
-      <c r="C202" s="8" t="s">
+      <c r="C201" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E201" s="2" t="s">
         <v>515</v>
       </c>
-      <c r="D202" s="8" t="s">
+    </row>
+    <row r="202" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A202" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="E202" s="8" t="s">
+      <c r="B202" s="2" t="s">
         <v>517</v>
+      </c>
+      <c r="C202" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D202" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E202" s="2" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A203" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="B203" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="C203" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D203" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E203" s="2" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A204" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B204" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="C204" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D204" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E204" s="2" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A205" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B205" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C205" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D205" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E205" s="2" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A206" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="B206" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="C206" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D206" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E206" s="2" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A208" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="B208" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="C208" s="8" t="s">
+        <v>533</v>
+      </c>
+      <c r="D208" s="8" t="s">
+        <v>534</v>
+      </c>
+      <c r="E208" s="8" t="s">
+        <v>535</v>
       </c>
     </row>
   </sheetData>

</xml_diff>